<commit_message>
refactor: unify partition grouping to loan_date-derived month
All three sheets now derive month from date_col (loan_date) via to_month():
- Sheet 1 partition_distribution: part_id → to_month(date_col)
- Sheet 3 backtest_effect: already used loan_date (no change)
- Sheet 3 bin_performance: part_id → to_month(date_col)

Also:
- to_month(): pd.to_datetime + strftime('%Y%m') for robust zero-padding
- partition_col removed from required validation
- date_col becomes the canonical source of monthly grouping

86 tests pass.
</commit_message>
<xml_diff>
--- a/sample_report.xlsx
+++ b/sample_report.xlsx
@@ -5778,7 +5778,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.0548</t>
+          <t>0.0373</t>
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
@@ -5841,7 +5841,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0.0753</t>
+          <t>0.0493</t>
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
@@ -5993,7 +5993,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>0.3482</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6055,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.1952</t>
+          <t>0.3184</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -6122,12 +6122,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>0.5088</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>0.1899</t>
         </is>
       </c>
     </row>
@@ -6189,12 +6189,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0.2601</t>
+          <t>inf</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>0.4089</t>
         </is>
       </c>
     </row>
@@ -6256,12 +6256,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>0.1652</t>
+          <t>inf</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>0.3315</t>
         </is>
       </c>
     </row>
@@ -6323,12 +6323,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>0.3521</t>
+          <t>inf</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>0.3301</t>
         </is>
       </c>
     </row>
@@ -6390,12 +6390,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>0.3666</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>0.1927</t>
+          <t>0.2809</t>
         </is>
       </c>
     </row>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>0.2355</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: calc_var_iv now correctly reads toad DataFrame output
Root cause: toad.quality() returns a DataFrame with 'iv' column
(vars as index), but calc_var_iv checked for pd.Series only and
fell through to float(DataFrame) which raised TypeError, caught
by except and silently returned 0.0.

Fix: check for pd.DataFrame first, extract value from 'iv' column.
Verified: iv_train now shows actual IV values (e.g., 1.12, 0.91).
</commit_message>
<xml_diff>
--- a/sample_report.xlsx
+++ b/sample_report.xlsx
@@ -1029,7 +1029,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -1037,7 +1037,7 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
@@ -1146,12 +1146,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1.53</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>rat1_sum_bu_1_14_pboc_aj65_cur</t>
+          <t>cu_ln_acct_lurate_gt50_arto</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -1189,37 +1189,37 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6.05%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.91</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>2.19</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0.29</t>
+          <t>0.33</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0.2245</t>
+          <t>0.0288</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>cu_ln_acct_lurate_gt50_arto</t>
+          <t>sum_bu_1_01_pboc_aa1_m12m</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -1252,27 +1252,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.81</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1.98</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>0.30</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.0288</t>
+          <t>0.2376</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>r24m_cfcbnkndpst_noacct_ln_tac</t>
+          <t>r12p24m_njslap_qtcnt</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -1290,7 +1290,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1305,27 +1305,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.67</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>2.26</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.11</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0.27</t>
+          <t>0.33</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0.0089</t>
+          <t>0.0952</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>sum_bu_1_01_pboc_aa1_m12m</t>
+          <t>agaa_zbvg_xavm_bbvf_mf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -1348,37 +1348,37 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>4.98%</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.63</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0.30</t>
+          <t>0.29</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>0.2376</t>
+          <t>0.1817</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>agaa_zbvg_xavm_bbvf_mf</t>
+          <t>rat1_sum_bu_1_14_pboc_aj65_cur</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -1401,27 +1401,27 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4.98%</t>
+          <t>6.05%</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>3.00%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.62</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>0.1817</t>
+          <t>0.2245</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>r12p24m_njslap_qtcnt</t>
+          <t>r24m_cfcbnkndpst_noacct_ln_tac</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -1449,7 +1449,7 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1464,27 +1464,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.21</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>0.11</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>0.27</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>0.0952</t>
+          <t>0.0089</t>
         </is>
       </c>
     </row>
@@ -2048,7 +2048,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>rat1_sum_bu_1_14_pboc_aj65_cur</t>
+          <t>cu_ln_acct_lurate_gt50_arto</t>
         </is>
       </c>
     </row>
@@ -2116,54 +2116,54 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>-999999.001</v>
+        <v>0.0061</v>
       </c>
       <c r="B27" t="n">
-        <v>0.0803</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="C27" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E27" t="n">
         <v>29</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>9.30%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>21.74%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>6.90%</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>0.8488</v>
+        <v>-0.1852</v>
       </c>
       <c r="J27" t="n">
-        <v>0.1056</v>
+        <v>0.0033</v>
       </c>
       <c r="K27" t="n">
-        <v>0.1244</v>
+        <v>0.0177</v>
       </c>
       <c r="L27" t="n">
-        <v>2.1064</v>
+        <v>0.8426</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.0803</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="B28" t="n">
-        <v>0.258</v>
+        <v>0.136</v>
       </c>
       <c r="C28" t="n">
         <v>25</v>
@@ -2204,98 +2204,98 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.258</v>
+        <v>0.136</v>
       </c>
       <c r="B29" t="n">
-        <v>0.471</v>
+        <v>0.179</v>
       </c>
       <c r="C29" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" t="n">
         <v>28</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>10.47%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>3.57%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>-0.8784</v>
+        <v>-0.1475</v>
       </c>
       <c r="J29" t="n">
-        <v>0.0537</v>
+        <v>0.002</v>
       </c>
       <c r="K29" t="n">
-        <v>0.0612</v>
+        <v>0.0138</v>
       </c>
       <c r="L29" t="n">
-        <v>0.4363</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0.471</v>
+        <v>0.179</v>
       </c>
       <c r="B30" t="n">
-        <v>0.669</v>
+        <v>0.226</v>
       </c>
       <c r="C30" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
         <v>28</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>-0.1475</v>
+        <v>-20.8051</v>
       </c>
       <c r="J30" t="n">
-        <v>0.002</v>
+        <v>2.2579</v>
       </c>
       <c r="K30" t="n">
-        <v>0.0138</v>
+        <v>0.1085</v>
       </c>
       <c r="L30" t="n">
-        <v>0.8727</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0.669</v>
+        <v>0.226</v>
       </c>
       <c r="B31" t="n">
-        <v>0.907</v>
+        <v>0.252</v>
       </c>
       <c r="C31" t="n">
         <v>26</v>
@@ -2336,142 +2336,142 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0.907</v>
+        <v>0.252</v>
       </c>
       <c r="B32" t="n">
-        <v>1.19</v>
+        <v>0.301</v>
       </c>
       <c r="C32" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E32" t="n">
         <v>28</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>9.30%</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>17.39%</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>14.29%</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>-0.1475</v>
+        <v>0.6257</v>
       </c>
       <c r="J32" t="n">
-        <v>0.002</v>
+        <v>0.0506</v>
       </c>
       <c r="K32" t="n">
-        <v>0.0138</v>
+        <v>0.0809</v>
       </c>
       <c r="L32" t="n">
-        <v>0.8727</v>
+        <v>1.7453</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1.19</v>
+        <v>0.301</v>
       </c>
       <c r="B33" t="n">
-        <v>1.36</v>
+        <v>0.356</v>
       </c>
       <c r="C33" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33" t="n">
         <v>28</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>-0.1475</v>
+        <v>-0.8784</v>
       </c>
       <c r="J33" t="n">
-        <v>0.002</v>
+        <v>0.0537</v>
       </c>
       <c r="K33" t="n">
-        <v>0.0138</v>
+        <v>0.0612</v>
       </c>
       <c r="L33" t="n">
-        <v>0.8727</v>
+        <v>0.4363</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1.36</v>
+        <v>0.356</v>
       </c>
       <c r="B34" t="n">
-        <v>1.561</v>
+        <v>0.419</v>
       </c>
       <c r="C34" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
         <v>28</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>-0.1475</v>
+        <v>-20.8051</v>
       </c>
       <c r="J34" t="n">
-        <v>0.002</v>
+        <v>2.2579</v>
       </c>
       <c r="K34" t="n">
-        <v>0.0138</v>
+        <v>0.1085</v>
       </c>
       <c r="L34" t="n">
-        <v>0.8727</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1.561</v>
+        <v>0.419</v>
       </c>
       <c r="B35" t="n">
-        <v>1.8</v>
+        <v>0.503</v>
       </c>
       <c r="C35" t="n">
         <v>25</v>
@@ -2512,46 +2512,46 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1.8</v>
+        <v>0.503</v>
       </c>
       <c r="B36" t="n">
-        <v>1.996</v>
+        <v>0.757</v>
       </c>
       <c r="C36" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E36" t="n">
         <v>28</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>10.47%</t>
+          <t>8.53%</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>26.09%</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>3.57%</t>
+          <t>21.43%</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>-0.8784</v>
+        <v>1.1182</v>
       </c>
       <c r="J36" t="n">
-        <v>0.0537</v>
+        <v>0.1964</v>
       </c>
       <c r="K36" t="n">
-        <v>0.0612</v>
+        <v>0.1756</v>
       </c>
       <c r="L36" t="n">
-        <v>0.4363</v>
+        <v>2.618</v>
       </c>
     </row>
     <row r="37">
@@ -2593,7 +2593,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>0.243</v>
+        <v>4.843799999999999</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -2605,7 +2605,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>cu_ln_acct_lurate_gt50_arto</t>
+          <t>sum_bu_1_01_pboc_aa1_m12m</t>
         </is>
       </c>
     </row>
@@ -2673,98 +2673,98 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0.0061</v>
+        <v>79724.999</v>
       </c>
       <c r="B41" t="n">
-        <v>0.09859999999999999</v>
+        <v>621650</v>
       </c>
       <c r="C41" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D41" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E41" t="n">
         <v>29</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>10.47%</t>
+          <t>9.30%</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>21.74%</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>6.90%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>-0.1852</v>
+        <v>0.8488</v>
       </c>
       <c r="J41" t="n">
-        <v>0.0033</v>
+        <v>0.1056</v>
       </c>
       <c r="K41" t="n">
-        <v>0.0177</v>
+        <v>0.1244</v>
       </c>
       <c r="L41" t="n">
-        <v>0.8426</v>
+        <v>2.1064</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0.09859999999999999</v>
+        <v>621650</v>
       </c>
       <c r="B42" t="n">
-        <v>0.136</v>
+        <v>1112636</v>
       </c>
       <c r="C42" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
         <v>28</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>0.2972</v>
+        <v>-0.8784</v>
       </c>
       <c r="J42" t="n">
-        <v>0.01</v>
+        <v>0.0537</v>
       </c>
       <c r="K42" t="n">
-        <v>0.0335</v>
+        <v>0.0612</v>
       </c>
       <c r="L42" t="n">
-        <v>1.309</v>
+        <v>0.4363</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>0.136</v>
+        <v>1112636</v>
       </c>
       <c r="B43" t="n">
-        <v>0.179</v>
+        <v>1625557</v>
       </c>
       <c r="C43" t="n">
         <v>26</v>
@@ -2805,230 +2805,230 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0.179</v>
+        <v>1625557</v>
       </c>
       <c r="B44" t="n">
-        <v>0.226</v>
+        <v>1928266</v>
       </c>
       <c r="C44" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E44" t="n">
         <v>28</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>9.30%</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>17.39%</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>14.29%</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>-20.8051</v>
+        <v>0.6257</v>
       </c>
       <c r="J44" t="n">
-        <v>2.2579</v>
+        <v>0.0506</v>
       </c>
       <c r="K44" t="n">
-        <v>0.1085</v>
+        <v>0.0809</v>
       </c>
       <c r="L44" t="n">
-        <v>0</v>
+        <v>1.7453</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>0.226</v>
+        <v>1928266</v>
       </c>
       <c r="B45" t="n">
-        <v>0.252</v>
+        <v>2305363</v>
       </c>
       <c r="C45" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E45" t="n">
         <v>28</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>-0.1475</v>
+        <v>-0.8784</v>
       </c>
       <c r="J45" t="n">
-        <v>0.002</v>
+        <v>0.0537</v>
       </c>
       <c r="K45" t="n">
-        <v>0.0138</v>
+        <v>0.0612</v>
       </c>
       <c r="L45" t="n">
-        <v>0.8727</v>
+        <v>0.4363</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>0.252</v>
+        <v>2305363</v>
       </c>
       <c r="B46" t="n">
-        <v>0.301</v>
+        <v>2818362</v>
       </c>
       <c r="C46" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E46" t="n">
         <v>28</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>9.30%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>17.39%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>14.29%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.6257</v>
+        <v>-0.1475</v>
       </c>
       <c r="J46" t="n">
-        <v>0.0506</v>
+        <v>0.002</v>
       </c>
       <c r="K46" t="n">
-        <v>0.0809</v>
+        <v>0.0138</v>
       </c>
       <c r="L46" t="n">
-        <v>1.7453</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>0.301</v>
+        <v>2818362</v>
       </c>
       <c r="B47" t="n">
-        <v>0.356</v>
+        <v>3430889</v>
       </c>
       <c r="C47" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E47" t="n">
         <v>28</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>10.47%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>3.57%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>-0.8784</v>
+        <v>-0.1475</v>
       </c>
       <c r="J47" t="n">
-        <v>0.0537</v>
+        <v>0.002</v>
       </c>
       <c r="K47" t="n">
-        <v>0.0612</v>
+        <v>0.0138</v>
       </c>
       <c r="L47" t="n">
-        <v>0.4363</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>0.356</v>
+        <v>3430889</v>
       </c>
       <c r="B48" t="n">
-        <v>0.419</v>
+        <v>3971451</v>
       </c>
       <c r="C48" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48" t="n">
         <v>28</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>-20.8051</v>
+        <v>-0.8784</v>
       </c>
       <c r="J48" t="n">
-        <v>2.2579</v>
+        <v>0.0537</v>
       </c>
       <c r="K48" t="n">
-        <v>0.1085</v>
+        <v>0.0612</v>
       </c>
       <c r="L48" t="n">
-        <v>0</v>
+        <v>0.4363</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>0.419</v>
+        <v>3971451</v>
       </c>
       <c r="B49" t="n">
-        <v>0.503</v>
+        <v>4477036</v>
       </c>
       <c r="C49" t="n">
         <v>25</v>
@@ -3069,46 +3069,46 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>0.503</v>
+        <v>4477036</v>
       </c>
       <c r="B50" t="n">
-        <v>0.757</v>
+        <v>4983594</v>
       </c>
       <c r="C50" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E50" t="n">
         <v>28</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>8.53%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>26.09%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>21.43%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>1.1182</v>
+        <v>-0.1475</v>
       </c>
       <c r="J50" t="n">
-        <v>0.1964</v>
+        <v>0.002</v>
       </c>
       <c r="K50" t="n">
-        <v>0.1756</v>
+        <v>0.0138</v>
       </c>
       <c r="L50" t="n">
-        <v>2.618</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="51">
@@ -3150,7 +3150,7 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>4.843799999999999</v>
+        <v>0.3353</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -3162,7 +3162,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>r24m_cfcbnkndpst_noacct_ln_tac</t>
+          <t>r12p24m_njslap_qtcnt</t>
         </is>
       </c>
     </row>
@@ -3233,256 +3233,315 @@
         <v>-0.001</v>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>0.106</v>
       </c>
       <c r="C55" t="n">
-        <v>185</v>
+        <v>27</v>
       </c>
       <c r="D55" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="E55" t="n">
-        <v>199</v>
+        <v>29</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>71.71%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>60.87%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>7.04%</t>
+          <t>6.90%</t>
         </is>
       </c>
       <c r="I55" t="n">
-        <v>-0.1638</v>
+        <v>-0.1852</v>
       </c>
       <c r="J55" t="n">
-        <v>0.0178</v>
+        <v>0.0033</v>
       </c>
       <c r="K55" t="n">
-        <v>0.1084</v>
+        <v>0.0177</v>
       </c>
       <c r="L55" t="n">
-        <v>0.8595</v>
+        <v>0.8426</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="B56" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="C56" t="n">
+        <v>25</v>
+      </c>
+      <c r="D56" t="n">
+        <v>3</v>
+      </c>
+      <c r="E56" t="n">
+        <v>28</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>9.69%</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>13.04%</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>10.71%</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>0.2972</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.0335</v>
+      </c>
+      <c r="L56" t="n">
+        <v>1.309</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="B57" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="C57" t="n">
+        <v>25</v>
+      </c>
+      <c r="D57" t="n">
+        <v>3</v>
+      </c>
+      <c r="E57" t="n">
+        <v>28</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>9.69%</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>13.04%</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>10.71%</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>0.2972</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0.0335</v>
+      </c>
+      <c r="L57" t="n">
+        <v>1.309</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="B58" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="C58" t="n">
+        <v>26</v>
+      </c>
+      <c r="D58" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" t="n">
+        <v>28</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>10.08%</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>8.70%</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>7.14%</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>-0.1475</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.0138</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0.8727</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="B59" t="n">
+        <v>0.503</v>
+      </c>
+      <c r="C59" t="n">
+        <v>27</v>
+      </c>
+      <c r="D59" t="n">
         <v>1</v>
       </c>
-      <c r="B56" t="n">
-        <v>2</v>
-      </c>
-      <c r="C56" t="n">
-        <v>73</v>
-      </c>
-      <c r="D56" t="n">
-        <v>9</v>
-      </c>
-      <c r="E56" t="n">
-        <v>82</v>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>28.29%</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>39.13%</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>10.98%</t>
-        </is>
-      </c>
-      <c r="I56" t="n">
-        <v>0.3242</v>
-      </c>
-      <c r="J56" t="n">
-        <v>0.0351</v>
-      </c>
-      <c r="K56" t="n">
-        <v>0.1084</v>
-      </c>
-      <c r="L56" t="n">
-        <v>1.3409</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>258</v>
-      </c>
-      <c r="D57" t="n">
-        <v>23</v>
-      </c>
-      <c r="E57" t="n">
-        <v>281</v>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>8.19%</t>
-        </is>
-      </c>
-      <c r="I57" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" t="n">
-        <v>0.0529</v>
-      </c>
-      <c r="K57" t="n">
-        <v>0</v>
-      </c>
-      <c r="L57" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="inlineStr">
-        <is>
-          <t>sum_bu_1_01_pboc_aa1_m12m</t>
-        </is>
+      <c r="E59" t="n">
+        <v>28</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>10.47%</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>4.35%</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>3.57%</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>-0.8784</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.0537</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.0612</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0.4363</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>goods</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>bads</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>good_prop</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>bad_prop</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>bad_rate</t>
-        </is>
-      </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>woe</t>
-        </is>
-      </c>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>iv</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>ks</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="inlineStr">
-        <is>
-          <t>lift</t>
-        </is>
+      <c r="A60" t="n">
+        <v>0.503</v>
+      </c>
+      <c r="B60" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="C60" t="n">
+        <v>25</v>
+      </c>
+      <c r="D60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E60" t="n">
+        <v>28</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>9.69%</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>13.04%</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>10.71%</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>0.2972</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0.0335</v>
+      </c>
+      <c r="L60" t="n">
+        <v>1.309</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>79724.999</v>
+        <v>0.59</v>
       </c>
       <c r="B61" t="n">
-        <v>621650</v>
+        <v>0.669</v>
       </c>
       <c r="C61" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D61" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>9.30%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>21.74%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>17.24%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="I61" t="n">
-        <v>0.8488</v>
+        <v>-0.8784</v>
       </c>
       <c r="J61" t="n">
-        <v>0.1056</v>
+        <v>0.0537</v>
       </c>
       <c r="K61" t="n">
-        <v>0.1244</v>
+        <v>0.0612</v>
       </c>
       <c r="L61" t="n">
-        <v>2.1064</v>
+        <v>0.4363</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>621650</v>
+        <v>0.669</v>
       </c>
       <c r="B62" t="n">
-        <v>1112636</v>
+        <v>0.789</v>
       </c>
       <c r="C62" t="n">
         <v>27</v>
@@ -3523,54 +3582,54 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1112636</v>
+        <v>0.789</v>
       </c>
       <c r="B63" t="n">
-        <v>1625557</v>
+        <v>0.872</v>
       </c>
       <c r="C63" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E63" t="n">
         <v>28</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>9.69%</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="I63" t="n">
-        <v>-0.1475</v>
+        <v>0.2972</v>
       </c>
       <c r="J63" t="n">
-        <v>0.002</v>
+        <v>0.01</v>
       </c>
       <c r="K63" t="n">
-        <v>0.0138</v>
+        <v>0.0335</v>
       </c>
       <c r="L63" t="n">
-        <v>0.8727</v>
+        <v>1.309</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1625557</v>
+        <v>0.872</v>
       </c>
       <c r="B64" t="n">
-        <v>1928266</v>
+        <v>0.992</v>
       </c>
       <c r="C64" t="n">
         <v>24</v>
@@ -3610,436 +3669,436 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="n">
-        <v>1928266</v>
-      </c>
-      <c r="B65" t="n">
-        <v>2305363</v>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
       </c>
       <c r="C65" t="n">
-        <v>27</v>
+        <v>258</v>
       </c>
       <c r="D65" t="n">
+        <v>23</v>
+      </c>
+      <c r="E65" t="n">
+        <v>281</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>8.19%</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0.257</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="n">
         <v>1</v>
       </c>
-      <c r="E65" t="n">
-        <v>28</v>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>10.47%</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>4.35%</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
-      </c>
-      <c r="I65" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J65" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K65" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L65" t="n">
-        <v>0.4363</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="n">
-        <v>2305363</v>
-      </c>
-      <c r="B66" t="n">
-        <v>2818362</v>
-      </c>
-      <c r="C66" t="n">
-        <v>26</v>
-      </c>
-      <c r="D66" t="n">
-        <v>2</v>
-      </c>
-      <c r="E66" t="n">
-        <v>28</v>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>10.08%</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>8.70%</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
-      </c>
-      <c r="I66" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J66" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K66" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L66" t="n">
-        <v>0.8727</v>
-      </c>
     </row>
     <row r="67">
-      <c r="A67" t="n">
-        <v>2818362</v>
-      </c>
-      <c r="B67" t="n">
-        <v>3430889</v>
-      </c>
-      <c r="C67" t="n">
-        <v>26</v>
-      </c>
-      <c r="D67" t="n">
-        <v>2</v>
-      </c>
-      <c r="E67" t="n">
-        <v>28</v>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>10.08%</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>8.70%</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
-      </c>
-      <c r="I67" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J67" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K67" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L67" t="n">
-        <v>0.8727</v>
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>agaa_zbvg_xavm_bbvf_mf</t>
+        </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="n">
-        <v>3430889</v>
-      </c>
-      <c r="B68" t="n">
-        <v>3971451</v>
-      </c>
-      <c r="C68" t="n">
-        <v>27</v>
-      </c>
-      <c r="D68" t="n">
-        <v>1</v>
-      </c>
-      <c r="E68" t="n">
-        <v>28</v>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>10.47%</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>4.35%</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
-      </c>
-      <c r="I68" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J68" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K68" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L68" t="n">
-        <v>0.4363</v>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>goods</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>bads</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>good_prop</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>bad_prop</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>bad_rate</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>woe</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>iv</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>lift</t>
+        </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>3971451</v>
+        <v>-999999.001</v>
       </c>
       <c r="B69" t="n">
-        <v>4477036</v>
+        <v>-802</v>
       </c>
       <c r="C69" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E69" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>3.45%</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>0.2972</v>
+        <v>-0.9147</v>
       </c>
       <c r="J69" t="n">
-        <v>0.01</v>
+        <v>0.0595</v>
       </c>
       <c r="K69" t="n">
-        <v>0.0335</v>
+        <v>0.065</v>
       </c>
       <c r="L69" t="n">
-        <v>1.309</v>
+        <v>0.4213</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>4477036</v>
+        <v>-802</v>
       </c>
       <c r="B70" t="n">
-        <v>4983594</v>
+        <v>-154</v>
       </c>
       <c r="C70" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E70" t="n">
         <v>28</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>9.69%</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>13.04%</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>10.71%</t>
         </is>
       </c>
       <c r="I70" t="n">
-        <v>-0.1475</v>
+        <v>0.2972</v>
       </c>
       <c r="J70" t="n">
-        <v>0.002</v>
+        <v>0.01</v>
       </c>
       <c r="K70" t="n">
-        <v>0.0138</v>
+        <v>0.0335</v>
       </c>
       <c r="L70" t="n">
-        <v>0.8727</v>
+        <v>1.309</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
+      <c r="A71" t="n">
+        <v>-154</v>
+      </c>
+      <c r="B71" t="n">
+        <v>297</v>
       </c>
       <c r="C71" t="n">
-        <v>258</v>
+        <v>24</v>
       </c>
       <c r="D71" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="E71" t="n">
-        <v>281</v>
+        <v>28</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>9.30%</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>17.39%</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>8.19%</t>
+          <t>14.29%</t>
         </is>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
+        <v>0.6257</v>
       </c>
       <c r="J71" t="n">
-        <v>0.3353</v>
+        <v>0.0506</v>
       </c>
       <c r="K71" t="n">
-        <v>0</v>
+        <v>0.0809</v>
       </c>
       <c r="L71" t="n">
-        <v>1</v>
+        <v>1.7453</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>297</v>
+      </c>
+      <c r="B72" t="n">
+        <v>610</v>
+      </c>
+      <c r="C72" t="n">
+        <v>28</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="n">
+        <v>28</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>10.85%</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>-20.8051</v>
+      </c>
+      <c r="J72" t="n">
+        <v>2.2579</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0.1085</v>
+      </c>
+      <c r="L72" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="inlineStr">
-        <is>
-          <t>agaa_zbvg_xavm_bbvf_mf</t>
-        </is>
+      <c r="A73" t="n">
+        <v>610</v>
+      </c>
+      <c r="B73" t="n">
+        <v>1004</v>
+      </c>
+      <c r="C73" t="n">
+        <v>25</v>
+      </c>
+      <c r="D73" t="n">
+        <v>3</v>
+      </c>
+      <c r="E73" t="n">
+        <v>28</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>9.69%</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>13.04%</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>10.71%</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>0.2972</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0.0335</v>
+      </c>
+      <c r="L73" t="n">
+        <v>1.309</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>goods</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>bads</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>good_prop</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>bad_prop</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>bad_rate</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>woe</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>iv</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr">
-        <is>
-          <t>ks</t>
-        </is>
-      </c>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>lift</t>
-        </is>
+      <c r="A74" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B74" t="n">
+        <v>1444</v>
+      </c>
+      <c r="C74" t="n">
+        <v>25</v>
+      </c>
+      <c r="D74" t="n">
+        <v>3</v>
+      </c>
+      <c r="E74" t="n">
+        <v>28</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>9.69%</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>13.04%</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>10.71%</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>0.2972</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0.0335</v>
+      </c>
+      <c r="L74" t="n">
+        <v>1.309</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>-999999.001</v>
+        <v>1444</v>
       </c>
       <c r="B75" t="n">
-        <v>-802</v>
+        <v>1884</v>
       </c>
       <c r="C75" t="n">
+        <v>26</v>
+      </c>
+      <c r="D75" t="n">
+        <v>2</v>
+      </c>
+      <c r="E75" t="n">
         <v>28</v>
       </c>
-      <c r="D75" t="n">
-        <v>1</v>
-      </c>
-      <c r="E75" t="n">
-        <v>29</v>
-      </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>3.45%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="I75" t="n">
-        <v>-0.9147</v>
+        <v>-0.1475</v>
       </c>
       <c r="J75" t="n">
-        <v>0.0595</v>
+        <v>0.002</v>
       </c>
       <c r="K75" t="n">
-        <v>0.065</v>
+        <v>0.0138</v>
       </c>
       <c r="L75" t="n">
-        <v>0.4213</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>-802</v>
+        <v>1884</v>
       </c>
       <c r="B76" t="n">
-        <v>-154</v>
+        <v>2337</v>
       </c>
       <c r="C76" t="n">
         <v>25</v>
@@ -4080,492 +4139,492 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>-154</v>
+        <v>2337</v>
       </c>
       <c r="B77" t="n">
-        <v>297</v>
+        <v>2655</v>
       </c>
       <c r="C77" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D77" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E77" t="n">
         <v>28</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>9.30%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>17.39%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>14.29%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="I77" t="n">
-        <v>0.6257</v>
+        <v>-0.1475</v>
       </c>
       <c r="J77" t="n">
-        <v>0.0506</v>
+        <v>0.002</v>
       </c>
       <c r="K77" t="n">
-        <v>0.0809</v>
+        <v>0.0138</v>
       </c>
       <c r="L77" t="n">
-        <v>1.7453</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>297</v>
+        <v>2655</v>
       </c>
       <c r="B78" t="n">
-        <v>610</v>
+        <v>2999</v>
       </c>
       <c r="C78" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D78" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E78" t="n">
         <v>28</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>10.85%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="I78" t="n">
-        <v>-20.8051</v>
+        <v>-0.1475</v>
       </c>
       <c r="J78" t="n">
-        <v>2.2579</v>
+        <v>0.002</v>
       </c>
       <c r="K78" t="n">
-        <v>0.1085</v>
+        <v>0.0138</v>
       </c>
       <c r="L78" t="n">
-        <v>0</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="n">
-        <v>610</v>
-      </c>
-      <c r="B79" t="n">
-        <v>1004</v>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
       </c>
       <c r="C79" t="n">
-        <v>25</v>
+        <v>258</v>
       </c>
       <c r="D79" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="E79" t="n">
-        <v>28</v>
+        <v>281</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>8.19%</t>
         </is>
       </c>
       <c r="I79" t="n">
-        <v>0.2972</v>
+        <v>0</v>
       </c>
       <c r="J79" t="n">
-        <v>0.01</v>
+        <v>2.414</v>
       </c>
       <c r="K79" t="n">
-        <v>0.0335</v>
+        <v>0</v>
       </c>
       <c r="L79" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>1004</v>
-      </c>
-      <c r="B80" t="n">
-        <v>1444</v>
-      </c>
-      <c r="C80" t="n">
-        <v>25</v>
-      </c>
-      <c r="D80" t="n">
-        <v>3</v>
-      </c>
-      <c r="E80" t="n">
-        <v>28</v>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>9.69%</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>13.04%</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
-      </c>
-      <c r="I80" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J80" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K80" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L80" t="n">
-        <v>1.309</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="n">
-        <v>1444</v>
-      </c>
-      <c r="B81" t="n">
-        <v>1884</v>
-      </c>
-      <c r="C81" t="n">
-        <v>26</v>
-      </c>
-      <c r="D81" t="n">
-        <v>2</v>
-      </c>
-      <c r="E81" t="n">
-        <v>28</v>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>10.08%</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>8.70%</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
-      </c>
-      <c r="I81" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J81" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K81" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L81" t="n">
-        <v>0.8727</v>
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>rat1_sum_bu_1_14_pboc_aj65_cur</t>
+        </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="n">
-        <v>1884</v>
-      </c>
-      <c r="B82" t="n">
-        <v>2337</v>
-      </c>
-      <c r="C82" t="n">
-        <v>25</v>
-      </c>
-      <c r="D82" t="n">
-        <v>3</v>
-      </c>
-      <c r="E82" t="n">
-        <v>28</v>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>9.69%</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>13.04%</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
-      </c>
-      <c r="I82" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J82" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K82" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L82" t="n">
-        <v>1.309</v>
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>goods</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>bads</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>good_prop</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>bad_prop</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>bad_rate</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>woe</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>iv</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>lift</t>
+        </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>2337</v>
+        <v>-999999.001</v>
       </c>
       <c r="B83" t="n">
-        <v>2655</v>
+        <v>0.0803</v>
       </c>
       <c r="C83" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D83" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E83" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>9.30%</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>21.74%</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>17.24%</t>
         </is>
       </c>
       <c r="I83" t="n">
-        <v>-0.1475</v>
+        <v>0.8488</v>
       </c>
       <c r="J83" t="n">
-        <v>0.002</v>
+        <v>0.1056</v>
       </c>
       <c r="K83" t="n">
-        <v>0.0138</v>
+        <v>0.1244</v>
       </c>
       <c r="L83" t="n">
-        <v>0.8727</v>
+        <v>2.1064</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>2655</v>
+        <v>0.0803</v>
       </c>
       <c r="B84" t="n">
-        <v>2999</v>
+        <v>0.258</v>
       </c>
       <c r="C84" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E84" t="n">
         <v>28</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
+          <t>9.69%</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>13.04%</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>10.71%</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>0.2972</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0.0335</v>
+      </c>
+      <c r="L84" t="n">
+        <v>1.309</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="B85" t="n">
+        <v>0.471</v>
+      </c>
+      <c r="C85" t="n">
+        <v>27</v>
+      </c>
+      <c r="D85" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" t="n">
+        <v>28</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>10.47%</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>4.35%</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>3.57%</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>-0.8784</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0.0537</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0.0612</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0.4363</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>0.471</v>
+      </c>
+      <c r="B86" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="C86" t="n">
+        <v>26</v>
+      </c>
+      <c r="D86" t="n">
+        <v>2</v>
+      </c>
+      <c r="E86" t="n">
+        <v>28</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
           <t>10.08%</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
+      <c r="G86" t="inlineStr">
         <is>
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="H86" t="inlineStr">
         <is>
           <t>7.14%</t>
         </is>
       </c>
-      <c r="I84" t="n">
+      <c r="I86" t="n">
         <v>-0.1475</v>
       </c>
-      <c r="J84" t="n">
+      <c r="J86" t="n">
         <v>0.002</v>
       </c>
-      <c r="K84" t="n">
+      <c r="K86" t="n">
         <v>0.0138</v>
       </c>
-      <c r="L84" t="n">
+      <c r="L86" t="n">
         <v>0.8727</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C85" t="n">
-        <v>258</v>
-      </c>
-      <c r="D85" t="n">
-        <v>23</v>
-      </c>
-      <c r="E85" t="n">
-        <v>281</v>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>8.19%</t>
-        </is>
-      </c>
-      <c r="I85" t="n">
-        <v>0</v>
-      </c>
-      <c r="J85" t="n">
-        <v>2.414</v>
-      </c>
-      <c r="K85" t="n">
-        <v>0</v>
-      </c>
-      <c r="L85" t="n">
-        <v>1</v>
-      </c>
-    </row>
     <row r="87">
-      <c r="A87" s="1" t="inlineStr">
-        <is>
-          <t>r12p24m_njslap_qtcnt</t>
-        </is>
+      <c r="A87" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="B87" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="C87" t="n">
+        <v>26</v>
+      </c>
+      <c r="D87" t="n">
+        <v>2</v>
+      </c>
+      <c r="E87" t="n">
+        <v>28</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>10.08%</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>8.70%</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>7.14%</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>-0.1475</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0.0138</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0.8727</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>goods</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>bads</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t>good_prop</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t>bad_prop</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr">
-        <is>
-          <t>bad_rate</t>
-        </is>
-      </c>
-      <c r="I88" s="2" t="inlineStr">
-        <is>
-          <t>woe</t>
-        </is>
-      </c>
-      <c r="J88" s="2" t="inlineStr">
-        <is>
-          <t>iv</t>
-        </is>
-      </c>
-      <c r="K88" s="2" t="inlineStr">
-        <is>
-          <t>ks</t>
-        </is>
-      </c>
-      <c r="L88" s="2" t="inlineStr">
-        <is>
-          <t>lift</t>
-        </is>
+      <c r="A88" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="B88" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="C88" t="n">
+        <v>26</v>
+      </c>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
+      <c r="E88" t="n">
+        <v>28</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>10.08%</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>8.70%</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>7.14%</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>-0.1475</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0.0138</v>
+      </c>
+      <c r="L88" t="n">
+        <v>0.8727</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>-0.001</v>
+        <v>1.19</v>
       </c>
       <c r="B89" t="n">
-        <v>0.106</v>
+        <v>1.36</v>
       </c>
       <c r="C89" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D89" t="n">
         <v>2</v>
       </c>
       <c r="E89" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>10.47%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4575,72 +4634,72 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>6.90%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="I89" t="n">
-        <v>-0.1852</v>
+        <v>-0.1475</v>
       </c>
       <c r="J89" t="n">
-        <v>0.0033</v>
+        <v>0.002</v>
       </c>
       <c r="K89" t="n">
-        <v>0.0177</v>
+        <v>0.0138</v>
       </c>
       <c r="L89" t="n">
-        <v>0.8426</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>0.106</v>
+        <v>1.36</v>
       </c>
       <c r="B90" t="n">
-        <v>0.213</v>
+        <v>1.561</v>
       </c>
       <c r="C90" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E90" t="n">
         <v>28</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>10.08%</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>7.14%</t>
         </is>
       </c>
       <c r="I90" t="n">
-        <v>0.2972</v>
+        <v>-0.1475</v>
       </c>
       <c r="J90" t="n">
-        <v>0.01</v>
+        <v>0.002</v>
       </c>
       <c r="K90" t="n">
-        <v>0.0335</v>
+        <v>0.0138</v>
       </c>
       <c r="L90" t="n">
-        <v>1.309</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>0.213</v>
+        <v>1.561</v>
       </c>
       <c r="B91" t="n">
-        <v>0.303</v>
+        <v>1.8</v>
       </c>
       <c r="C91" t="n">
         <v>25</v>
@@ -4681,310 +4740,251 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0.303</v>
+        <v>1.8</v>
       </c>
       <c r="B92" t="n">
-        <v>0.418</v>
+        <v>1.996</v>
       </c>
       <c r="C92" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E92" t="n">
         <v>28</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>10.08%</t>
+          <t>10.47%</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>7.14%</t>
+          <t>3.57%</t>
         </is>
       </c>
       <c r="I92" t="n">
-        <v>-0.1475</v>
+        <v>-0.8784</v>
       </c>
       <c r="J92" t="n">
-        <v>0.002</v>
+        <v>0.0537</v>
       </c>
       <c r="K92" t="n">
-        <v>0.0138</v>
+        <v>0.0612</v>
       </c>
       <c r="L92" t="n">
-        <v>0.8727</v>
+        <v>0.4363</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="n">
-        <v>0.418</v>
-      </c>
-      <c r="B93" t="n">
-        <v>0.503</v>
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
       </c>
       <c r="C93" t="n">
-        <v>27</v>
+        <v>258</v>
       </c>
       <c r="D93" t="n">
+        <v>23</v>
+      </c>
+      <c r="E93" t="n">
+        <v>281</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>8.19%</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
         <v>1</v>
       </c>
-      <c r="E93" t="n">
-        <v>28</v>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>10.47%</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>4.35%</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
-      </c>
-      <c r="I93" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J93" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K93" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L93" t="n">
-        <v>0.4363</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>0.503</v>
-      </c>
-      <c r="B94" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="C94" t="n">
-        <v>25</v>
-      </c>
-      <c r="D94" t="n">
-        <v>3</v>
-      </c>
-      <c r="E94" t="n">
-        <v>28</v>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>9.69%</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>13.04%</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
-      </c>
-      <c r="I94" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J94" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K94" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L94" t="n">
-        <v>1.309</v>
-      </c>
     </row>
     <row r="95">
-      <c r="A95" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="B95" t="n">
-        <v>0.669</v>
-      </c>
-      <c r="C95" t="n">
-        <v>27</v>
-      </c>
-      <c r="D95" t="n">
-        <v>1</v>
-      </c>
-      <c r="E95" t="n">
-        <v>28</v>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>10.47%</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>4.35%</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
-      </c>
-      <c r="I95" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J95" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K95" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L95" t="n">
-        <v>0.4363</v>
+      <c r="A95" s="1" t="inlineStr">
+        <is>
+          <t>r24m_cfcbnkndpst_noacct_ln_tac</t>
+        </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="n">
-        <v>0.669</v>
-      </c>
-      <c r="B96" t="n">
-        <v>0.789</v>
-      </c>
-      <c r="C96" t="n">
-        <v>27</v>
-      </c>
-      <c r="D96" t="n">
-        <v>1</v>
-      </c>
-      <c r="E96" t="n">
-        <v>28</v>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>10.47%</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>4.35%</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
-      </c>
-      <c r="I96" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J96" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K96" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L96" t="n">
-        <v>0.4363</v>
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>goods</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>bads</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>good_prop</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>bad_prop</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>bad_rate</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>woe</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>iv</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>lift</t>
+        </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>0.789</v>
+        <v>-0.001</v>
       </c>
       <c r="B97" t="n">
-        <v>0.872</v>
+        <v>1</v>
       </c>
       <c r="C97" t="n">
-        <v>25</v>
+        <v>185</v>
       </c>
       <c r="D97" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="E97" t="n">
-        <v>28</v>
+        <v>199</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>9.69%</t>
+          <t>71.71%</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>13.04%</t>
+          <t>60.87%</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>10.71%</t>
+          <t>7.04%</t>
         </is>
       </c>
       <c r="I97" t="n">
-        <v>0.2972</v>
+        <v>-0.1638</v>
       </c>
       <c r="J97" t="n">
-        <v>0.01</v>
+        <v>0.0178</v>
       </c>
       <c r="K97" t="n">
-        <v>0.0335</v>
+        <v>0.1084</v>
       </c>
       <c r="L97" t="n">
-        <v>1.309</v>
+        <v>0.8595</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>0.872</v>
+        <v>1</v>
       </c>
       <c r="B98" t="n">
-        <v>0.992</v>
+        <v>2</v>
       </c>
       <c r="C98" t="n">
-        <v>24</v>
+        <v>73</v>
       </c>
       <c r="D98" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>9.30%</t>
+          <t>28.29%</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>17.39%</t>
+          <t>39.13%</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>14.29%</t>
+          <t>10.98%</t>
         </is>
       </c>
       <c r="I98" t="n">
-        <v>0.6257</v>
+        <v>0.3242</v>
       </c>
       <c r="J98" t="n">
-        <v>0.0506</v>
+        <v>0.0351</v>
       </c>
       <c r="K98" t="n">
-        <v>0.0809</v>
+        <v>0.1084</v>
       </c>
       <c r="L98" t="n">
-        <v>1.7453</v>
+        <v>1.3409</v>
       </c>
     </row>
     <row r="99">
@@ -5026,7 +5026,7 @@
         <v>0</v>
       </c>
       <c r="J99" t="n">
-        <v>0.257</v>
+        <v>0.0529</v>
       </c>
       <c r="K99" t="n">
         <v>0</v>
@@ -5117,7 +5117,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H55:H57">
+  <conditionalFormatting sqref="H55:H65">
     <cfRule type="dataBar" priority="10">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5126,7 +5126,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I55:I57">
+  <conditionalFormatting sqref="I55:I65">
     <cfRule type="dataBar" priority="11">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5135,7 +5135,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L55:L57">
+  <conditionalFormatting sqref="L55:L65">
     <cfRule type="dataBar" priority="12">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5144,7 +5144,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H61:H71">
+  <conditionalFormatting sqref="H69:H79">
     <cfRule type="dataBar" priority="13">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5153,7 +5153,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I61:I71">
+  <conditionalFormatting sqref="I69:I79">
     <cfRule type="dataBar" priority="14">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5162,7 +5162,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L61:L71">
+  <conditionalFormatting sqref="L69:L79">
     <cfRule type="dataBar" priority="15">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5171,7 +5171,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H75:H85">
+  <conditionalFormatting sqref="H83:H93">
     <cfRule type="dataBar" priority="16">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5180,7 +5180,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I75:I85">
+  <conditionalFormatting sqref="I83:I93">
     <cfRule type="dataBar" priority="17">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5189,7 +5189,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L75:L85">
+  <conditionalFormatting sqref="L83:L93">
     <cfRule type="dataBar" priority="18">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5198,7 +5198,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H89:H99">
+  <conditionalFormatting sqref="H97:H99">
     <cfRule type="dataBar" priority="19">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5207,7 +5207,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I89:I99">
+  <conditionalFormatting sqref="I97:I99">
     <cfRule type="dataBar" priority="20">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -5216,7 +5216,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L89:L99">
+  <conditionalFormatting sqref="L97:L99">
     <cfRule type="dataBar" priority="21">
       <dataBar showValue="1">
         <cfvo type="min"/>

</xml_diff>

<commit_message>
fix: WOE table — bad_rate numeric for data bars, iv/ks/lift 2dp
- bad_rate kept as numeric (not percentage string) for data bar rendering
- iv/ks/lift precision changed from 4dp to 2dp in compute_woe_table
- good_prop/bad_prop remain as formatted percentage strings
</commit_message>
<xml_diff>
--- a/sample_report.xlsx
+++ b/sample_report.xlsx
@@ -1042,11 +1042,11 @@
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -1590,22 +1590,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>3.45%</t>
-        </is>
+      <c r="H13" s="3" t="n">
+        <v>0.0345</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>-0.9147</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.0595</v>
+        <v>0.06</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0.065</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>0.4213</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="14">
@@ -1634,22 +1632,20 @@
           <t>26.09%</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>20.00%</t>
-        </is>
+      <c r="H14" s="3" t="n">
+        <v>0.2</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>1.0312</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.1731</v>
+        <v>0.17</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0.1678</v>
+        <v>0.17</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>2.4435</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="15">
@@ -1678,22 +1674,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>6.67%</t>
-        </is>
+      <c r="H15" s="3" t="n">
+        <v>0.0667</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>-0.2216</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.0048</v>
+        <v>0</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>0.0216</v>
+        <v>0.02</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>0.8145</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -1722,22 +1716,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>4.00%</t>
-        </is>
+      <c r="H16" s="3" t="n">
+        <v>0.04</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>-0.7606000000000001</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.0377</v>
+        <v>0.04</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0.0495</v>
+        <v>0.05</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0.4887</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="17">
@@ -1766,22 +1758,20 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
+      <c r="H17" s="3" t="n">
+        <v>0.1</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>0.2202</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.0057</v>
+        <v>0.01</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0.0258</v>
+        <v>0.03</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>1.2217</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="18">
@@ -1810,19 +1800,17 @@
           <t>17.39%</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>14.81%</t>
-        </is>
+      <c r="H18" s="3" t="n">
+        <v>0.1481</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>0.6683</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.0566</v>
+        <v>0.06</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0.0848</v>
+        <v>0.08</v>
       </c>
       <c r="L18" s="3" t="n">
         <v>1.81</v>
@@ -1854,22 +1842,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H19" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="20">
@@ -1898,22 +1884,20 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>11.11%</t>
-        </is>
+      <c r="H20" s="3" t="n">
+        <v>0.1111</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>0.338</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.0126</v>
+        <v>0.01</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>0.0374</v>
+        <v>0.04</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>1.3575</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="21">
@@ -1942,22 +1926,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>3.33%</t>
-        </is>
+      <c r="H21" s="3" t="n">
+        <v>0.0333</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>-0.9498</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.0655</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0.0689</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>0.4072</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="22">
@@ -1986,19 +1968,17 @@
           <t>0.00%</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
+      <c r="H22" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>-20.6918</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>2.005</v>
+        <v>2.01</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>0.0969</v>
+        <v>0.1</v>
       </c>
       <c r="L22" s="3" t="n">
         <v>0</v>
@@ -2034,16 +2014,14 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>8.19%</t>
-        </is>
+      <c r="H23" s="3" t="n">
+        <v>0.08185053380782918</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>2.4225</v>
+        <v>2.43</v>
       </c>
       <c r="K23" s="3" t="n">
         <v>0</v>
@@ -2147,22 +2125,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>6.90%</t>
-        </is>
+      <c r="H27" s="3" t="n">
+        <v>0.06900000000000001</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>-0.1852</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.0033</v>
+        <v>0</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>0.0177</v>
+        <v>0.02</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>0.8426</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="28">
@@ -2191,10 +2167,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H28" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>0.2972</v>
@@ -2203,10 +2177,10 @@
         <v>0.01</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="29">
@@ -2235,22 +2209,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H29" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="30">
@@ -2279,19 +2251,17 @@
           <t>0.00%</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
+      <c r="H30" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>-20.8051</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>2.2579</v>
+        <v>2.26</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0.1085</v>
+        <v>0.11</v>
       </c>
       <c r="L30" s="3" t="n">
         <v>0</v>
@@ -2323,22 +2293,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H31" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="32">
@@ -2367,22 +2335,20 @@
           <t>17.39%</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>14.29%</t>
-        </is>
+      <c r="H32" s="3" t="n">
+        <v>0.1429</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>0.6257</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.0506</v>
+        <v>0.05</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>0.0809</v>
+        <v>0.08</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>1.7453</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="33">
@@ -2411,22 +2377,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
+      <c r="H33" s="3" t="n">
+        <v>0.0357</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>-0.8784</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.05</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.06</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.4363</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="34">
@@ -2455,19 +2419,17 @@
           <t>0.00%</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
+      <c r="H34" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>-20.8051</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>2.2579</v>
+        <v>2.26</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.1085</v>
+        <v>0.11</v>
       </c>
       <c r="L34" s="3" t="n">
         <v>0</v>
@@ -2499,10 +2461,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H35" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>0.2972</v>
@@ -2511,10 +2471,10 @@
         <v>0.01</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="36">
@@ -2543,22 +2503,20 @@
           <t>26.09%</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>21.43%</t>
-        </is>
+      <c r="H36" s="3" t="n">
+        <v>0.2143</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>1.1182</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.1964</v>
+        <v>0.2</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.1756</v>
+        <v>0.18</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>2.618</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="37">
@@ -2591,16 +2549,14 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>8.19%</t>
-        </is>
+      <c r="H37" s="3" t="n">
+        <v>0.08185053380782918</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>4.843799999999999</v>
+        <v>4.839999999999999</v>
       </c>
       <c r="K37" s="3" t="n">
         <v>0</v>
@@ -2704,22 +2660,20 @@
           <t>21.74%</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>17.24%</t>
-        </is>
+      <c r="H41" s="3" t="n">
+        <v>0.1724</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>0.8488</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.1056</v>
+        <v>0.11</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0.1244</v>
+        <v>0.12</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>2.1064</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="42">
@@ -2748,22 +2702,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
+      <c r="H42" s="3" t="n">
+        <v>0.0357</v>
       </c>
       <c r="I42" s="3" t="n">
         <v>-0.8784</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.05</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.06</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>0.4363</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="43">
@@ -2792,22 +2744,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H43" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I43" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="44">
@@ -2836,22 +2786,20 @@
           <t>17.39%</t>
         </is>
       </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>14.29%</t>
-        </is>
+      <c r="H44" s="3" t="n">
+        <v>0.1429</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>0.6257</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.0506</v>
+        <v>0.05</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0.0809</v>
+        <v>0.08</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>1.7453</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="45">
@@ -2880,22 +2828,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
+      <c r="H45" s="3" t="n">
+        <v>0.0357</v>
       </c>
       <c r="I45" s="3" t="n">
         <v>-0.8784</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.05</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.06</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>0.4363</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="46">
@@ -2924,22 +2870,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H46" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I46" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="47">
@@ -2968,22 +2912,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H47" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="48">
@@ -3012,22 +2954,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
+      <c r="H48" s="3" t="n">
+        <v>0.0357</v>
       </c>
       <c r="I48" s="3" t="n">
         <v>-0.8784</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.05</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.06</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>0.4363</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="49">
@@ -3056,10 +2996,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H49" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I49" s="3" t="n">
         <v>0.2972</v>
@@ -3068,10 +3006,10 @@
         <v>0.01</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="50">
@@ -3100,22 +3038,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H50" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I50" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L50" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="51">
@@ -3148,16 +3084,14 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr">
-        <is>
-          <t>8.19%</t>
-        </is>
+      <c r="H51" s="3" t="n">
+        <v>0.08185053380782918</v>
       </c>
       <c r="I51" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>0.3353</v>
+        <v>0.3200000000000001</v>
       </c>
       <c r="K51" s="3" t="n">
         <v>0</v>
@@ -3261,22 +3195,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>6.90%</t>
-        </is>
+      <c r="H55" s="3" t="n">
+        <v>0.06900000000000001</v>
       </c>
       <c r="I55" s="3" t="n">
         <v>-0.1852</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>0.0033</v>
+        <v>0</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>0.0177</v>
+        <v>0.02</v>
       </c>
       <c r="L55" s="3" t="n">
-        <v>0.8426</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="56">
@@ -3305,10 +3237,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H56" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H56" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I56" s="3" t="n">
         <v>0.2972</v>
@@ -3317,10 +3247,10 @@
         <v>0.01</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L56" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="57">
@@ -3349,10 +3279,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H57" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I57" s="3" t="n">
         <v>0.2972</v>
@@ -3361,10 +3289,10 @@
         <v>0.01</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L57" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="58">
@@ -3393,22 +3321,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H58" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I58" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L58" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="59">
@@ -3437,22 +3363,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
+      <c r="H59" s="3" t="n">
+        <v>0.0357</v>
       </c>
       <c r="I59" s="3" t="n">
         <v>-0.8784</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.05</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.06</v>
       </c>
       <c r="L59" s="3" t="n">
-        <v>0.4363</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="60">
@@ -3481,10 +3405,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H60" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I60" s="3" t="n">
         <v>0.2972</v>
@@ -3493,10 +3415,10 @@
         <v>0.01</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L60" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="61">
@@ -3525,22 +3447,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
+      <c r="H61" s="3" t="n">
+        <v>0.0357</v>
       </c>
       <c r="I61" s="3" t="n">
         <v>-0.8784</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.05</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.06</v>
       </c>
       <c r="L61" s="3" t="n">
-        <v>0.4363</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="62">
@@ -3569,22 +3489,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H62" s="3" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
+      <c r="H62" s="3" t="n">
+        <v>0.0357</v>
       </c>
       <c r="I62" s="3" t="n">
         <v>-0.8784</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.05</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.06</v>
       </c>
       <c r="L62" s="3" t="n">
-        <v>0.4363</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="63">
@@ -3613,10 +3531,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H63" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I63" s="3" t="n">
         <v>0.2972</v>
@@ -3625,10 +3541,10 @@
         <v>0.01</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L63" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="64">
@@ -3657,22 +3573,20 @@
           <t>17.39%</t>
         </is>
       </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>14.29%</t>
-        </is>
+      <c r="H64" s="3" t="n">
+        <v>0.1429</v>
       </c>
       <c r="I64" s="3" t="n">
         <v>0.6257</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>0.0506</v>
+        <v>0.05</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>0.0809</v>
+        <v>0.08</v>
       </c>
       <c r="L64" s="3" t="n">
-        <v>1.7453</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="65">
@@ -3705,16 +3619,14 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="H65" s="3" t="inlineStr">
-        <is>
-          <t>8.19%</t>
-        </is>
+      <c r="H65" s="3" t="n">
+        <v>0.08185053380782918</v>
       </c>
       <c r="I65" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>0.257</v>
+        <v>0.24</v>
       </c>
       <c r="K65" s="3" t="n">
         <v>0</v>
@@ -3818,22 +3730,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H69" s="3" t="inlineStr">
-        <is>
-          <t>3.45%</t>
-        </is>
+      <c r="H69" s="3" t="n">
+        <v>0.0345</v>
       </c>
       <c r="I69" s="3" t="n">
         <v>-0.9147</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>0.0595</v>
+        <v>0.06</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>0.065</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="L69" s="3" t="n">
-        <v>0.4213</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="70">
@@ -3862,10 +3772,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H70" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I70" s="3" t="n">
         <v>0.2972</v>
@@ -3874,10 +3782,10 @@
         <v>0.01</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L70" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="71">
@@ -3906,22 +3814,20 @@
           <t>17.39%</t>
         </is>
       </c>
-      <c r="H71" s="3" t="inlineStr">
-        <is>
-          <t>14.29%</t>
-        </is>
+      <c r="H71" s="3" t="n">
+        <v>0.1429</v>
       </c>
       <c r="I71" s="3" t="n">
         <v>0.6257</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>0.0506</v>
+        <v>0.05</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>0.0809</v>
+        <v>0.08</v>
       </c>
       <c r="L71" s="3" t="n">
-        <v>1.7453</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="72">
@@ -3950,19 +3856,17 @@
           <t>0.00%</t>
         </is>
       </c>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
+      <c r="H72" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="I72" s="3" t="n">
         <v>-20.8051</v>
       </c>
       <c r="J72" s="3" t="n">
-        <v>2.2579</v>
+        <v>2.26</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>0.1085</v>
+        <v>0.11</v>
       </c>
       <c r="L72" s="3" t="n">
         <v>0</v>
@@ -3994,10 +3898,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H73" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H73" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I73" s="3" t="n">
         <v>0.2972</v>
@@ -4006,10 +3908,10 @@
         <v>0.01</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L73" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="74">
@@ -4038,10 +3940,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H74" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H74" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I74" s="3" t="n">
         <v>0.2972</v>
@@ -4050,10 +3950,10 @@
         <v>0.01</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L74" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="75">
@@ -4082,22 +3982,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H75" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H75" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I75" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J75" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L75" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="76">
@@ -4126,10 +4024,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H76" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H76" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I76" s="3" t="n">
         <v>0.2972</v>
@@ -4138,10 +4034,10 @@
         <v>0.01</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L76" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="77">
@@ -4170,22 +4066,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H77" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H77" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I77" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L77" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="78">
@@ -4214,22 +4108,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H78" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H78" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I78" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L78" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="79">
@@ -4262,16 +4154,14 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>8.19%</t>
-        </is>
+      <c r="H79" s="3" t="n">
+        <v>0.08185053380782918</v>
       </c>
       <c r="I79" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>2.414</v>
+        <v>2.409999999999999</v>
       </c>
       <c r="K79" s="3" t="n">
         <v>0</v>
@@ -4375,22 +4265,20 @@
           <t>21.74%</t>
         </is>
       </c>
-      <c r="H83" s="3" t="inlineStr">
-        <is>
-          <t>17.24%</t>
-        </is>
+      <c r="H83" s="3" t="n">
+        <v>0.1724</v>
       </c>
       <c r="I83" s="3" t="n">
         <v>0.8488</v>
       </c>
       <c r="J83" s="3" t="n">
-        <v>0.1056</v>
+        <v>0.11</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>0.1244</v>
+        <v>0.12</v>
       </c>
       <c r="L83" s="3" t="n">
-        <v>2.1064</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="84">
@@ -4419,10 +4307,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H84" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H84" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I84" s="3" t="n">
         <v>0.2972</v>
@@ -4431,10 +4317,10 @@
         <v>0.01</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L84" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="85">
@@ -4463,22 +4349,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H85" s="3" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
+      <c r="H85" s="3" t="n">
+        <v>0.0357</v>
       </c>
       <c r="I85" s="3" t="n">
         <v>-0.8784</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.05</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.06</v>
       </c>
       <c r="L85" s="3" t="n">
-        <v>0.4363</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="86">
@@ -4507,22 +4391,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H86" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H86" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I86" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L86" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="87">
@@ -4551,22 +4433,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H87" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H87" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I87" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J87" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L87" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="88">
@@ -4595,22 +4475,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H88" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H88" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I88" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J88" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L88" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="89">
@@ -4639,22 +4517,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H89" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H89" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I89" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L89" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="90">
@@ -4683,22 +4559,20 @@
           <t>8.70%</t>
         </is>
       </c>
-      <c r="H90" s="3" t="inlineStr">
-        <is>
-          <t>7.14%</t>
-        </is>
+      <c r="H90" s="3" t="n">
+        <v>0.07140000000000001</v>
       </c>
       <c r="I90" s="3" t="n">
         <v>-0.1475</v>
       </c>
       <c r="J90" s="3" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>0.0138</v>
+        <v>0.01</v>
       </c>
       <c r="L90" s="3" t="n">
-        <v>0.8727</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="91">
@@ -4727,10 +4601,8 @@
           <t>13.04%</t>
         </is>
       </c>
-      <c r="H91" s="3" t="inlineStr">
-        <is>
-          <t>10.71%</t>
-        </is>
+      <c r="H91" s="3" t="n">
+        <v>0.1071</v>
       </c>
       <c r="I91" s="3" t="n">
         <v>0.2972</v>
@@ -4739,10 +4611,10 @@
         <v>0.01</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>0.0335</v>
+        <v>0.03</v>
       </c>
       <c r="L91" s="3" t="n">
-        <v>1.309</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="92">
@@ -4771,22 +4643,20 @@
           <t>4.35%</t>
         </is>
       </c>
-      <c r="H92" s="3" t="inlineStr">
-        <is>
-          <t>3.57%</t>
-        </is>
+      <c r="H92" s="3" t="n">
+        <v>0.0357</v>
       </c>
       <c r="I92" s="3" t="n">
         <v>-0.8784</v>
       </c>
       <c r="J92" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.05</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>0.0612</v>
+        <v>0.06</v>
       </c>
       <c r="L92" s="3" t="n">
-        <v>0.4363</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="93">
@@ -4819,16 +4689,14 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="H93" s="3" t="inlineStr">
-        <is>
-          <t>8.19%</t>
-        </is>
+      <c r="H93" s="3" t="n">
+        <v>0.08185053380782918</v>
       </c>
       <c r="I93" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J93" s="3" t="n">
-        <v>0.243</v>
+        <v>0.23</v>
       </c>
       <c r="K93" s="3" t="n">
         <v>0</v>
@@ -4932,22 +4800,20 @@
           <t>60.87%</t>
         </is>
       </c>
-      <c r="H97" s="3" t="inlineStr">
-        <is>
-          <t>7.04%</t>
-        </is>
+      <c r="H97" s="3" t="n">
+        <v>0.0704</v>
       </c>
       <c r="I97" s="3" t="n">
         <v>-0.1638</v>
       </c>
       <c r="J97" s="3" t="n">
-        <v>0.0178</v>
+        <v>0.02</v>
       </c>
       <c r="K97" s="3" t="n">
-        <v>0.1084</v>
+        <v>0.11</v>
       </c>
       <c r="L97" s="3" t="n">
-        <v>0.8595</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="98">
@@ -4976,22 +4842,20 @@
           <t>39.13%</t>
         </is>
       </c>
-      <c r="H98" s="3" t="inlineStr">
-        <is>
-          <t>10.98%</t>
-        </is>
+      <c r="H98" s="3" t="n">
+        <v>0.1098</v>
       </c>
       <c r="I98" s="3" t="n">
         <v>0.3242</v>
       </c>
       <c r="J98" s="3" t="n">
-        <v>0.0351</v>
+        <v>0.04</v>
       </c>
       <c r="K98" s="3" t="n">
-        <v>0.1084</v>
+        <v>0.11</v>
       </c>
       <c r="L98" s="3" t="n">
-        <v>1.3409</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="99">
@@ -5024,16 +4888,14 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="H99" s="3" t="inlineStr">
-        <is>
-          <t>8.19%</t>
-        </is>
+      <c r="H99" s="3" t="n">
+        <v>0.08185053380782918</v>
       </c>
       <c r="I99" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J99" s="3" t="n">
-        <v>0.0529</v>
+        <v>0.06</v>
       </c>
       <c r="K99" s="3" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
style: all cells center-aligned, CJK-aware column auto-fit
- Data cells: horizontal center + vertical center
- Section titles: left-aligned, vertical center
- Column width: CJK characters counted as 2x width vs ASCII 1x
- Max column width capped at 45 chars

90 tests pass.
</commit_message>
<xml_diff>
--- a/sample_report.xlsx
+++ b/sample_report.xlsx
@@ -71,11 +71,15 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,12 +448,12 @@
   <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1035,19 +1039,19 @@
   <dimension ref="A1:M99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5107,21 +5111,21 @@
   <dimension ref="A1:O181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
fix: data bar color with alpha prefix (FF5B9BD5 → fully opaque)
</commit_message>
<xml_diff>
--- a/sample_report.xlsx
+++ b/sample_report.xlsx
@@ -4653,7 +4653,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4662,7 +4662,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4671,7 +4671,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4680,7 +4680,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4689,7 +4689,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4698,7 +4698,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4707,7 +4707,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4716,7 +4716,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4725,7 +4725,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4734,7 +4734,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4743,7 +4743,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4752,7 +4752,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4761,7 +4761,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4770,7 +4770,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4779,7 +4779,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4788,7 +4788,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4797,7 +4797,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4806,7 +4806,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4815,7 +4815,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4824,7 +4824,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -4833,7 +4833,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11038,7 +11038,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11047,7 +11047,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11056,7 +11056,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11065,7 +11065,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11074,7 +11074,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11083,7 +11083,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11092,7 +11092,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11101,7 +11101,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11110,7 +11110,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11119,7 +11119,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11128,7 +11128,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11137,7 +11137,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11146,7 +11146,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11155,7 +11155,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11164,7 +11164,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11173,7 +11173,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11182,7 +11182,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11191,7 +11191,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11200,7 +11200,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11209,7 +11209,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11218,7 +11218,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11227,7 +11227,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11236,7 +11236,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11245,7 +11245,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11254,7 +11254,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11263,7 +11263,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11272,7 +11272,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11281,7 +11281,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11290,7 +11290,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11299,7 +11299,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11308,7 +11308,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11317,7 +11317,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11326,7 +11326,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11335,7 +11335,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11344,7 +11344,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11353,7 +11353,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11362,7 +11362,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11371,7 +11371,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11380,7 +11380,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11389,7 +11389,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11398,7 +11398,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11407,7 +11407,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11416,7 +11416,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11425,7 +11425,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11434,7 +11434,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11443,7 +11443,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11452,7 +11452,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11461,7 +11461,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11470,7 +11470,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11479,7 +11479,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11488,7 +11488,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11497,7 +11497,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11506,7 +11506,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11515,7 +11515,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11524,7 +11524,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>
@@ -11533,7 +11533,7 @@
       <dataBar showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
-        <color rgb="005B9BD5"/>
+        <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat: monotonic WOE binning with missing value handling
Replace simple qcut with full monotonic binning from dataset_learn.py:
1. Separate MISSING_VALUE bin (NaN + <= -99999)
2. Fine 20-bin percentile binning
3. Proportion-constrained merging (3%-50% per bin)
4. WOE monotonicity enforcement (increase)
5. Target count reduction (merge by WOE gap, ≤6 bins)
6. Final monotonicity re-check (iterative)
7. ALL summary row appended

Categorical variables: one bin per unique value (no merging).
Fallback: simple 5-bin qcut if monotonic merge fails.

94 tests pass.
</commit_message>
<xml_diff>
--- a/sample_report.xlsx
+++ b/sample_report.xlsx
@@ -1051,10 +1051,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M99"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
@@ -1584,780 +1584,712 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
-        <v>0.999</v>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
       </c>
       <c r="B13" s="3" t="n">
         <v>6</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.1085271317829457</v>
+        <v>0.09302325581395349</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.04347826086956522</v>
+        <v>0</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.0345</v>
+        <v>0</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>-0.9147</v>
+        <v>-20.6509</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0.0595</v>
+        <v>1.921</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>0.065</v>
+        <v>0.093</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>0.4213</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B14" s="3" t="n">
-        <v>12</v>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>24</v>
+        <v>234</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>30</v>
+        <v>257</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.09302325581395349</v>
+        <v>0.9069767441860465</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>0.2608695652173913</v>
+        <v>1</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0.2</v>
+        <v>0.0895</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>1.0312</v>
+        <v>0.09760000000000001</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>0.1731</v>
+        <v>0.0091</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>0.1678</v>
+        <v>0.093</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>2.4435</v>
+        <v>1.0934</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>19</v>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>28</v>
+        <v>258</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>30</v>
+        <v>281</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.1085271317829457</v>
+        <v>1</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.08695652173913043</v>
+        <v>1</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.0667</v>
+        <v>0.08185053380782918</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>-0.2216</v>
+        <v>0</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.0048</v>
+        <v>1.9301</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>0.0216</v>
+        <v>0</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>0.8145</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D16" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>0.09302325581395349</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="I16" s="6" t="n">
-        <v>-0.7606000000000001</v>
-      </c>
-      <c r="J16" s="6" t="n">
-        <v>0.0377</v>
-      </c>
-      <c r="K16" s="6" t="n">
-        <v>0.0495</v>
-      </c>
-      <c r="L16" s="6" t="n">
-        <v>0.4887</v>
-      </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I17" s="6" t="n">
-        <v>0.2202</v>
-      </c>
-      <c r="J17" s="6" t="n">
-        <v>0.0057</v>
-      </c>
-      <c r="K17" s="6" t="n">
-        <v>0.0258</v>
-      </c>
-      <c r="L17" s="6" t="n">
-        <v>1.2217</v>
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>cu_ln_acct_lurate_gt50_arto</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>37</v>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>0.08914728682170543</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>0.1739130434782609</v>
-      </c>
-      <c r="H18" s="4" t="n">
-        <v>0.1481</v>
-      </c>
-      <c r="I18" s="6" t="n">
-        <v>0.6683</v>
-      </c>
-      <c r="J18" s="6" t="n">
-        <v>0.0566</v>
-      </c>
-      <c r="K18" s="6" t="n">
-        <v>0.0848</v>
-      </c>
-      <c r="L18" s="6" t="n">
-        <v>1.81</v>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>goods</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>bads</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>good_prop</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>bad_prop</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>bad_rate</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>woe</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>iv</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>lift</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>37</v>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>44</v>
+        <v>0.2255</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>28</v>
+        <v>112</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.1007751937984496</v>
+        <v>0.4069767441860465</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.08695652173913043</v>
+        <v>0.3043478260869565</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.0625</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>-0.1475</v>
+        <v>-0.2906</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>0.002</v>
+        <v>0.0298</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>0.0138</v>
+        <v>0.1026</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>0.8727</v>
+        <v>0.7635999999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>44</v>
+        <v>0.2255</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>49</v>
+        <v>0.4194</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>24</v>
+        <v>105</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>27</v>
+        <v>112</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.09302325581395349</v>
+        <v>0.4069767441860465</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>0.1304347826086956</v>
+        <v>0.3043478260869565</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.1111</v>
+        <v>0.0625</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.338</v>
+        <v>-0.2906</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>0.0126</v>
+        <v>0.0298</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0.0374</v>
+        <v>0.1026</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>1.3575</v>
+        <v>0.7635999999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>49</v>
+        <v>0.4194</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>54</v>
+        <v>0.455</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.1124031007751938</v>
+        <v>0.05038759689922481</v>
       </c>
       <c r="G21" s="5" t="n">
         <v>0.04347826086956522</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>0.0333</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>-0.9498</v>
+        <v>-0.1475</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0.0655</v>
+        <v>0.001</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0.0689</v>
+        <v>0.0069</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>0.4072</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>54</v>
+        <v>0.455</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>59</v>
+        <v>0.5027</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.09689922480620156</v>
+        <v>0.04651162790697674</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>0</v>
+        <v>0.08695652173913043</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0</v>
+        <v>0.1429</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>-20.6918</v>
+        <v>0.6257</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>2.005</v>
+        <v>0.0253</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>0.0969</v>
+        <v>0.0404</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>0</v>
+        <v>1.7453</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="3" t="n">
+        <v>0.5027</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0.08914728682170543</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0.2608695652173913</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0.2069</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>1.0737</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>0.1844</v>
+      </c>
+      <c r="K23" s="6" t="n">
+        <v>0.1717</v>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>2.5277</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C24" s="3" t="n">
         <v>258</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D24" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E24" s="3" t="n">
         <v>281</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="G24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="4" t="n">
+      <c r="H24" s="4" t="n">
         <v>0.08185053380782918</v>
       </c>
-      <c r="I23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="6" t="n">
-        <v>2.4225</v>
-      </c>
-      <c r="K23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="6" t="n">
+      <c r="I24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>0.2703</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="6" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>cu_ln_acct_lurate_gt50_arto</t>
-        </is>
-      </c>
-    </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>sum_bu_1_01_pboc_aa1_m12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>max</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>goods</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>bads</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>good_prop</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>bad_prop</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>bad_rate</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>woe</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>iv</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>lift</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="n">
-        <v>0.0061</v>
-      </c>
-      <c r="B27" s="3" t="n">
-        <v>0.09859999999999999</v>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H27" s="4" t="n">
-        <v>0.06900000000000001</v>
-      </c>
-      <c r="I27" s="6" t="n">
-        <v>-0.1852</v>
-      </c>
-      <c r="J27" s="6" t="n">
-        <v>0.0033</v>
-      </c>
-      <c r="K27" s="6" t="n">
-        <v>0.0177</v>
-      </c>
-      <c r="L27" s="6" t="n">
-        <v>0.8426</v>
-      </c>
-    </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
-        <v>0.09859999999999999</v>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>0.136</v>
+        <v>4189289</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>25</v>
+        <v>220</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>28</v>
+        <v>238</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.09689922480620156</v>
+        <v>0.8527131782945736</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>0.1304347826086956</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.0756</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>0.2972</v>
+        <v>-0.0858</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
       <c r="K28" s="6" t="n">
-        <v>0.0335</v>
+        <v>0.0701</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>1.309</v>
+        <v>0.924</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>0.136</v>
-      </c>
-      <c r="B29" s="3" t="n">
-        <v>0.179</v>
+        <v>4189289</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.1007751937984496</v>
+        <v>0.1472868217054264</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>0.08695652173913043</v>
+        <v>0.2173913043478261</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.1163</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>-0.1475</v>
+        <v>0.3893</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>0.002</v>
+        <v>0.0273</v>
       </c>
       <c r="K29" s="6" t="n">
-        <v>0.0138</v>
+        <v>0.0701</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>0.8727</v>
+        <v>1.4206</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
-        <v>0.179</v>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>0.226</v>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>28</v>
+        <v>258</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>28</v>
+        <v>281</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.1085271317829457</v>
+        <v>1</v>
       </c>
       <c r="G30" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>0</v>
+        <v>0.08185053380782918</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>-20.8051</v>
+        <v>0</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>2.2579</v>
+        <v>0.0333</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>0.1085</v>
+        <v>0</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="n">
-        <v>0.226</v>
-      </c>
-      <c r="B31" s="3" t="n">
-        <v>0.252</v>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G31" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H31" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I31" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J31" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K31" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L31" s="6" t="n">
-        <v>0.8727</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
-        <v>0.252</v>
-      </c>
-      <c r="B32" s="3" t="n">
-        <v>0.301</v>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F32" s="5" t="n">
-        <v>0.09302325581395349</v>
-      </c>
-      <c r="G32" s="5" t="n">
-        <v>0.1739130434782609</v>
-      </c>
-      <c r="H32" s="4" t="n">
-        <v>0.1429</v>
-      </c>
-      <c r="I32" s="6" t="n">
-        <v>0.6257</v>
-      </c>
-      <c r="J32" s="6" t="n">
-        <v>0.0506</v>
-      </c>
-      <c r="K32" s="6" t="n">
-        <v>0.0809</v>
-      </c>
-      <c r="L32" s="6" t="n">
-        <v>1.7453</v>
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>r12p24m_njslap_qtcnt</t>
+        </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
-        <v>0.301</v>
-      </c>
-      <c r="B33" s="3" t="n">
-        <v>0.356</v>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F33" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G33" s="5" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H33" s="4" t="n">
-        <v>0.0357</v>
-      </c>
-      <c r="I33" s="6" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J33" s="6" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K33" s="6" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L33" s="6" t="n">
-        <v>0.4363</v>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>goods</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>bads</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>good_prop</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>bad_prop</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>bad_rate</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>woe</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>iv</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>lift</t>
+        </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
-        <v>0.356</v>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>0.419</v>
+        <v>0.0566</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.1085271317829457</v>
+        <v>0.05426356589147287</v>
       </c>
       <c r="G34" s="5" t="n">
         <v>0</v>
@@ -2366,13 +2298,13 @@
         <v>0</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>-20.8051</v>
+        <v>-20.1119</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>2.2579</v>
+        <v>1.0913</v>
       </c>
       <c r="K34" s="6" t="n">
-        <v>0.1085</v>
+        <v>0.0543</v>
       </c>
       <c r="L34" s="6" t="n">
         <v>0</v>
@@ -2380,2275 +2312,895 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>0.419</v>
+        <v>0.0566</v>
       </c>
       <c r="B35" s="3" t="n">
-        <v>0.503</v>
+        <v>0.7886</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>25</v>
+        <v>194</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>28</v>
+        <v>210</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.09689922480620156</v>
+        <v>0.751937984496124</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>0.1304347826086956</v>
+        <v>0.6956521739130435</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.0762</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>0.2972</v>
+        <v>-0.07779999999999999</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>0.01</v>
+        <v>0.0044</v>
       </c>
       <c r="K35" s="6" t="n">
-        <v>0.0335</v>
+        <v>0.0563</v>
       </c>
       <c r="L35" s="6" t="n">
-        <v>1.309</v>
+        <v>0.9308</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>0.503</v>
+        <v>0.7886</v>
       </c>
       <c r="B36" s="3" t="n">
-        <v>0.757</v>
+        <v>0.9352</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.08527131782945736</v>
+        <v>0.1472868217054264</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.1739130434782609</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>0.2143</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>1.1182</v>
+        <v>0.1662</v>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0.1964</v>
+        <v>0.0044</v>
       </c>
       <c r="K36" s="6" t="n">
-        <v>0.1756</v>
+        <v>0.0266</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>2.618</v>
+        <v>1.1636</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="3" t="n">
+        <v>0.9352</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>0.04651162790697674</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>0.1304347826086956</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I37" s="6" t="n">
+        <v>1.0312</v>
+      </c>
+      <c r="J37" s="6" t="n">
+        <v>0.08649999999999999</v>
+      </c>
+      <c r="K37" s="6" t="n">
+        <v>0.0839</v>
+      </c>
+      <c r="L37" s="6" t="n">
+        <v>2.4435</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C38" s="3" t="n">
         <v>258</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D38" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="E37" s="3" t="n">
+      <c r="E38" s="3" t="n">
         <v>281</v>
       </c>
-      <c r="F37" s="5" t="n">
+      <c r="F38" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G37" s="5" t="n">
+      <c r="G38" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H37" s="4" t="n">
+      <c r="H38" s="4" t="n">
         <v>0.08185053380782918</v>
       </c>
-      <c r="I37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" s="6" t="n">
-        <v>4.843799999999999</v>
-      </c>
-      <c r="K37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" s="6" t="n">
+      <c r="I38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="6" t="n">
+        <v>1.1866</v>
+      </c>
+      <c r="K38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="6" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
-        <is>
-          <t>sum_bu_1_01_pboc_aa1_m12m</t>
-        </is>
-      </c>
-    </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>agaa_zbvg_xavm_bbvf_mf</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>max</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>goods</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>bads</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>good_prop</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>bad_prop</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>bad_rate</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>woe</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>iv</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>lift</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="3" t="n">
-        <v>79724.999</v>
-      </c>
-      <c r="B41" s="3" t="n">
-        <v>621650</v>
-      </c>
-      <c r="C41" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D41" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E41" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="F41" s="5" t="n">
-        <v>0.09302325581395349</v>
-      </c>
-      <c r="G41" s="5" t="n">
-        <v>0.2173913043478261</v>
-      </c>
-      <c r="H41" s="4" t="n">
-        <v>0.1724</v>
-      </c>
-      <c r="I41" s="6" t="n">
-        <v>0.8488</v>
-      </c>
-      <c r="J41" s="6" t="n">
-        <v>0.1056</v>
-      </c>
-      <c r="K41" s="6" t="n">
-        <v>0.1244</v>
-      </c>
-      <c r="L41" s="6" t="n">
-        <v>2.1064</v>
-      </c>
-    </row>
     <row r="42">
-      <c r="A42" s="3" t="n">
-        <v>621650</v>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>1112636</v>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_VALUE</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_VALUE</t>
+        </is>
       </c>
       <c r="C42" s="3" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="D42" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.1046511627906977</v>
+        <v>0.05038759689922481</v>
       </c>
       <c r="G42" s="5" t="n">
         <v>0.04347826086956522</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0.0357</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="I42" s="6" t="n">
-        <v>-0.8784</v>
+        <v>-0.1475</v>
       </c>
       <c r="J42" s="6" t="n">
-        <v>0.0537</v>
+        <v>0.001</v>
       </c>
       <c r="K42" s="6" t="n">
-        <v>0.0612</v>
+        <v>0.0069</v>
       </c>
       <c r="L42" s="6" t="n">
-        <v>0.4363</v>
+        <v>0.8727</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n">
-        <v>1112636</v>
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>1625557</v>
+        <v>-804.8</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>0.1007751937984496</v>
+        <v>0.05426356589147287</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>0.08695652173913043</v>
+        <v>0</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>0.07140000000000001</v>
+        <v>0</v>
       </c>
       <c r="I43" s="6" t="n">
-        <v>-0.1475</v>
+        <v>-20.1119</v>
       </c>
       <c r="J43" s="6" t="n">
-        <v>0.002</v>
+        <v>1.0913</v>
       </c>
       <c r="K43" s="6" t="n">
-        <v>0.0138</v>
+        <v>0.0543</v>
       </c>
       <c r="L43" s="6" t="n">
-        <v>0.8727</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
-        <v>1625557</v>
+        <v>-804.8</v>
       </c>
       <c r="B44" s="3" t="n">
-        <v>1928266</v>
+        <v>-432</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.09302325581395349</v>
+        <v>0.04651162790697674</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>0.1739130434782609</v>
+        <v>0.04347826086956522</v>
       </c>
       <c r="H44" s="4" t="n">
-        <v>0.1429</v>
+        <v>0.0769</v>
       </c>
       <c r="I44" s="6" t="n">
-        <v>0.6257</v>
+        <v>-0.0674</v>
       </c>
       <c r="J44" s="6" t="n">
-        <v>0.0506</v>
+        <v>0.0002</v>
       </c>
       <c r="K44" s="6" t="n">
-        <v>0.0809</v>
+        <v>0.003</v>
       </c>
       <c r="L44" s="6" t="n">
-        <v>1.7453</v>
+        <v>0.9398</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
-        <v>1928266</v>
+        <v>-432</v>
       </c>
       <c r="B45" s="3" t="n">
-        <v>2305363</v>
+        <v>1942.2</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>27</v>
+        <v>146</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.1046511627906977</v>
+        <v>0.5658914728682171</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>0.04347826086956522</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>0.0357</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="I45" s="6" t="n">
-        <v>-0.8784</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="J45" s="6" t="n">
-        <v>0.0537</v>
+        <v>0.0031</v>
       </c>
       <c r="K45" s="6" t="n">
-        <v>0.0612</v>
+        <v>0.0428</v>
       </c>
       <c r="L45" s="6" t="n">
-        <v>0.4363</v>
+        <v>1.069</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
-        <v>2305363</v>
-      </c>
-      <c r="B46" s="3" t="n">
-        <v>2818362</v>
+        <v>1942.2</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0.1007751937984496</v>
+        <v>0.2829457364341085</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0.08695652173913043</v>
+        <v>0.3043478260869565</v>
       </c>
       <c r="H46" s="4" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="I46" s="6" t="n">
-        <v>-0.1475</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="J46" s="6" t="n">
-        <v>0.002</v>
+        <v>0.0016</v>
       </c>
       <c r="K46" s="6" t="n">
-        <v>0.0138</v>
+        <v>0.0214</v>
       </c>
       <c r="L46" s="6" t="n">
-        <v>0.8727</v>
+        <v>1.069</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="n">
-        <v>2818362</v>
-      </c>
-      <c r="B47" s="3" t="n">
-        <v>3430889</v>
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>26</v>
+        <v>258</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>28</v>
+        <v>281</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.1007751937984496</v>
+        <v>1</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>0.08695652173913043</v>
+        <v>1</v>
       </c>
       <c r="H47" s="4" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.08185053380782918</v>
       </c>
       <c r="I47" s="6" t="n">
-        <v>-0.1475</v>
+        <v>0</v>
       </c>
       <c r="J47" s="6" t="n">
-        <v>0.002</v>
+        <v>1.0972</v>
       </c>
       <c r="K47" s="6" t="n">
-        <v>0.0138</v>
+        <v>0</v>
       </c>
       <c r="L47" s="6" t="n">
-        <v>0.8727</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="n">
-        <v>3430889</v>
-      </c>
-      <c r="B48" s="3" t="n">
-        <v>3971451</v>
-      </c>
-      <c r="C48" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D48" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E48" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F48" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G48" s="5" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H48" s="4" t="n">
-        <v>0.0357</v>
-      </c>
-      <c r="I48" s="6" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J48" s="6" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K48" s="6" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L48" s="6" t="n">
-        <v>0.4363</v>
-      </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="n">
-        <v>3971451</v>
-      </c>
-      <c r="B49" s="3" t="n">
-        <v>4477036</v>
-      </c>
-      <c r="C49" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E49" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F49" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G49" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H49" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I49" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J49" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K49" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L49" s="6" t="n">
-        <v>1.309</v>
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>rat1_sum_bu_1_14_pboc_aj65_cur</t>
+        </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="n">
-        <v>4477036</v>
-      </c>
-      <c r="B50" s="3" t="n">
-        <v>4983594</v>
-      </c>
-      <c r="C50" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D50" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E50" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F50" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G50" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H50" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I50" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J50" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K50" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L50" s="6" t="n">
-        <v>0.8727</v>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>goods</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>bads</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>good_prop</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>bad_prop</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>bad_rate</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>woe</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>iv</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>lift</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
+          <t>MISSING_VALUE</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_VALUE</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>0.05813953488372093</v>
+      </c>
+      <c r="G51" s="5" t="n">
+        <v>0.08695652173913043</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>0.1176</v>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>0.4026</v>
+      </c>
+      <c r="J51" s="6" t="n">
+        <v>0.0116</v>
+      </c>
+      <c r="K51" s="6" t="n">
+        <v>0.0288</v>
+      </c>
+      <c r="L51" s="6" t="n">
+        <v>1.4373</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1.479045</v>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>183</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>198</v>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>0.7093023255813954</v>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>0.6521739130434783</v>
+      </c>
+      <c r="H52" s="4" t="n">
+        <v>0.07580000000000001</v>
+      </c>
+      <c r="I52" s="6" t="n">
+        <v>-0.08400000000000001</v>
+      </c>
+      <c r="J52" s="6" t="n">
+        <v>0.0048</v>
+      </c>
+      <c r="K52" s="6" t="n">
+        <v>0.0571</v>
+      </c>
+      <c r="L52" s="6" t="n">
+        <v>0.9256</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>1.479045</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>0.2325581395348837</v>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>0.2608695652173913</v>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>0.09089999999999999</v>
+      </c>
+      <c r="I53" s="6" t="n">
+        <v>0.1149</v>
+      </c>
+      <c r="J53" s="6" t="n">
+        <v>0.0033</v>
+      </c>
+      <c r="K53" s="6" t="n">
+        <v>0.0283</v>
+      </c>
+      <c r="L53" s="6" t="n">
+        <v>1.1107</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>
       </c>
-      <c r="C51" s="3" t="n">
+      <c r="C54" s="3" t="n">
         <v>258</v>
       </c>
-      <c r="D51" s="3" t="n">
+      <c r="D54" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="E51" s="3" t="n">
+      <c r="E54" s="3" t="n">
         <v>281</v>
       </c>
-      <c r="F51" s="5" t="n">
+      <c r="F54" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G51" s="5" t="n">
+      <c r="G54" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H51" s="4" t="n">
+      <c r="H54" s="4" t="n">
         <v>0.08185053380782918</v>
       </c>
-      <c r="I51" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" s="6" t="n">
-        <v>0.3353</v>
-      </c>
-      <c r="K51" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" s="6" t="n">
+      <c r="I54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="6" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="K54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="6" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="1" t="inlineStr">
-        <is>
-          <t>r12p24m_njslap_qtcnt</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>r24m_cfcbnkndpst_noacct_ln_tac</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>max</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>goods</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>bads</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>good_prop</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>bad_prop</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>bad_rate</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>woe</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="J57" s="2" t="inlineStr">
         <is>
           <t>iv</t>
         </is>
       </c>
-      <c r="K54" s="2" t="inlineStr">
+      <c r="K57" s="2" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
+      <c r="L57" s="2" t="inlineStr">
         <is>
           <t>lift</t>
         </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="n">
-        <v>-0.001</v>
-      </c>
-      <c r="B55" s="3" t="n">
-        <v>0.106</v>
-      </c>
-      <c r="C55" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D55" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E55" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="F55" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G55" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H55" s="4" t="n">
-        <v>0.06900000000000001</v>
-      </c>
-      <c r="I55" s="6" t="n">
-        <v>-0.1852</v>
-      </c>
-      <c r="J55" s="6" t="n">
-        <v>0.0033</v>
-      </c>
-      <c r="K55" s="6" t="n">
-        <v>0.0177</v>
-      </c>
-      <c r="L55" s="6" t="n">
-        <v>0.8426</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="n">
-        <v>0.106</v>
-      </c>
-      <c r="B56" s="3" t="n">
-        <v>0.213</v>
-      </c>
-      <c r="C56" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D56" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E56" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F56" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G56" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H56" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I56" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J56" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K56" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L56" s="6" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="n">
-        <v>0.213</v>
-      </c>
-      <c r="B57" s="3" t="n">
-        <v>0.303</v>
-      </c>
-      <c r="C57" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D57" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E57" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F57" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G57" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H57" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I57" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J57" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K57" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L57" s="6" t="n">
-        <v>1.309</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
-        <v>0.303</v>
+        <v>0</v>
       </c>
       <c r="B58" s="3" t="n">
-        <v>0.418</v>
+        <v>2</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>26</v>
+        <v>185</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>28</v>
+        <v>199</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>0.1007751937984496</v>
+        <v>0.7170542635658915</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>0.08695652173913043</v>
+        <v>0.6086956521739131</v>
       </c>
       <c r="H58" s="4" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.0704</v>
       </c>
       <c r="I58" s="6" t="n">
-        <v>-0.1475</v>
+        <v>-0.1638</v>
       </c>
       <c r="J58" s="6" t="n">
-        <v>0.002</v>
+        <v>0.0178</v>
       </c>
       <c r="K58" s="6" t="n">
-        <v>0.0138</v>
+        <v>0.1084</v>
       </c>
       <c r="L58" s="6" t="n">
-        <v>0.8727</v>
+        <v>0.8595</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
-        <v>0.418</v>
-      </c>
-      <c r="B59" s="3" t="n">
-        <v>0.503</v>
+        <v>2</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="C59" s="3" t="n">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="D59" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="F59" s="5" t="n">
+        <v>0.2829457364341085</v>
+      </c>
+      <c r="G59" s="5" t="n">
+        <v>0.391304347826087</v>
+      </c>
+      <c r="H59" s="4" t="n">
+        <v>0.1098</v>
+      </c>
+      <c r="I59" s="6" t="n">
+        <v>0.3242</v>
+      </c>
+      <c r="J59" s="6" t="n">
+        <v>0.0351</v>
+      </c>
+      <c r="K59" s="6" t="n">
+        <v>0.1084</v>
+      </c>
+      <c r="L59" s="6" t="n">
+        <v>1.3409</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>281</v>
+      </c>
+      <c r="F60" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E59" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F59" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G59" s="5" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H59" s="4" t="n">
-        <v>0.0357</v>
-      </c>
-      <c r="I59" s="6" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J59" s="6" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K59" s="6" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L59" s="6" t="n">
-        <v>0.4363</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="n">
-        <v>0.503</v>
-      </c>
-      <c r="B60" s="3" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="C60" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D60" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E60" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F60" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
       <c r="G60" s="5" t="n">
-        <v>0.1304347826086956</v>
+        <v>1</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>0.1071</v>
+        <v>0.08185053380782918</v>
       </c>
       <c r="I60" s="6" t="n">
-        <v>0.2972</v>
+        <v>0</v>
       </c>
       <c r="J60" s="6" t="n">
-        <v>0.01</v>
+        <v>0.0529</v>
       </c>
       <c r="K60" s="6" t="n">
-        <v>0.0335</v>
+        <v>0</v>
       </c>
       <c r="L60" s="6" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="B61" s="3" t="n">
-        <v>0.669</v>
-      </c>
-      <c r="C61" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D61" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E61" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F61" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G61" s="5" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H61" s="4" t="n">
-        <v>0.0357</v>
-      </c>
-      <c r="I61" s="6" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J61" s="6" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K61" s="6" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L61" s="6" t="n">
-        <v>0.4363</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="n">
-        <v>0.669</v>
-      </c>
-      <c r="B62" s="3" t="n">
-        <v>0.789</v>
-      </c>
-      <c r="C62" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D62" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F62" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G62" s="5" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H62" s="4" t="n">
-        <v>0.0357</v>
-      </c>
-      <c r="I62" s="6" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J62" s="6" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K62" s="6" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L62" s="6" t="n">
-        <v>0.4363</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="n">
-        <v>0.789</v>
-      </c>
-      <c r="B63" s="3" t="n">
-        <v>0.872</v>
-      </c>
-      <c r="C63" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D63" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E63" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F63" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G63" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H63" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I63" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J63" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K63" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L63" s="6" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="n">
-        <v>0.872</v>
-      </c>
-      <c r="B64" s="3" t="n">
-        <v>0.992</v>
-      </c>
-      <c r="C64" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D64" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E64" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F64" s="5" t="n">
-        <v>0.09302325581395349</v>
-      </c>
-      <c r="G64" s="5" t="n">
-        <v>0.1739130434782609</v>
-      </c>
-      <c r="H64" s="4" t="n">
-        <v>0.1429</v>
-      </c>
-      <c r="I64" s="6" t="n">
-        <v>0.6257</v>
-      </c>
-      <c r="J64" s="6" t="n">
-        <v>0.0506</v>
-      </c>
-      <c r="K64" s="6" t="n">
-        <v>0.0809</v>
-      </c>
-      <c r="L64" s="6" t="n">
-        <v>1.7453</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="n">
-        <v>258</v>
-      </c>
-      <c r="D65" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="E65" s="3" t="n">
-        <v>281</v>
-      </c>
-      <c r="F65" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G65" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H65" s="4" t="n">
-        <v>0.08185053380782918</v>
-      </c>
-      <c r="I65" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="6" t="n">
-        <v>0.257</v>
-      </c>
-      <c r="K65" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L65" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="inlineStr">
-        <is>
-          <t>agaa_zbvg_xavm_bbvf_mf</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>goods</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>bads</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>good_prop</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>bad_prop</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>bad_rate</t>
-        </is>
-      </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>woe</t>
-        </is>
-      </c>
-      <c r="J68" s="2" t="inlineStr">
-        <is>
-          <t>iv</t>
-        </is>
-      </c>
-      <c r="K68" s="2" t="inlineStr">
-        <is>
-          <t>ks</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="inlineStr">
-        <is>
-          <t>lift</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="n">
-        <v>-999999.001</v>
-      </c>
-      <c r="B69" s="3" t="n">
-        <v>-802</v>
-      </c>
-      <c r="C69" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="D69" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E69" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="F69" s="5" t="n">
-        <v>0.1085271317829457</v>
-      </c>
-      <c r="G69" s="5" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H69" s="4" t="n">
-        <v>0.0345</v>
-      </c>
-      <c r="I69" s="6" t="n">
-        <v>-0.9147</v>
-      </c>
-      <c r="J69" s="6" t="n">
-        <v>0.0595</v>
-      </c>
-      <c r="K69" s="6" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="L69" s="6" t="n">
-        <v>0.4213</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="n">
-        <v>-802</v>
-      </c>
-      <c r="B70" s="3" t="n">
-        <v>-154</v>
-      </c>
-      <c r="C70" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D70" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E70" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F70" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G70" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H70" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I70" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J70" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K70" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L70" s="6" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="n">
-        <v>-154</v>
-      </c>
-      <c r="B71" s="3" t="n">
-        <v>297</v>
-      </c>
-      <c r="C71" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D71" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E71" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F71" s="5" t="n">
-        <v>0.09302325581395349</v>
-      </c>
-      <c r="G71" s="5" t="n">
-        <v>0.1739130434782609</v>
-      </c>
-      <c r="H71" s="4" t="n">
-        <v>0.1429</v>
-      </c>
-      <c r="I71" s="6" t="n">
-        <v>0.6257</v>
-      </c>
-      <c r="J71" s="6" t="n">
-        <v>0.0506</v>
-      </c>
-      <c r="K71" s="6" t="n">
-        <v>0.0809</v>
-      </c>
-      <c r="L71" s="6" t="n">
-        <v>1.7453</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="n">
-        <v>297</v>
-      </c>
-      <c r="B72" s="3" t="n">
-        <v>610</v>
-      </c>
-      <c r="C72" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="D72" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E72" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F72" s="5" t="n">
-        <v>0.1085271317829457</v>
-      </c>
-      <c r="G72" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H72" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I72" s="6" t="n">
-        <v>-20.8051</v>
-      </c>
-      <c r="J72" s="6" t="n">
-        <v>2.2579</v>
-      </c>
-      <c r="K72" s="6" t="n">
-        <v>0.1085</v>
-      </c>
-      <c r="L72" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="3" t="n">
-        <v>610</v>
-      </c>
-      <c r="B73" s="3" t="n">
-        <v>1004</v>
-      </c>
-      <c r="C73" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D73" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E73" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F73" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G73" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H73" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I73" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J73" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K73" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L73" s="6" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="3" t="n">
-        <v>1004</v>
-      </c>
-      <c r="B74" s="3" t="n">
-        <v>1444</v>
-      </c>
-      <c r="C74" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D74" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E74" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F74" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G74" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H74" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I74" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J74" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K74" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L74" s="6" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="3" t="n">
-        <v>1444</v>
-      </c>
-      <c r="B75" s="3" t="n">
-        <v>1884</v>
-      </c>
-      <c r="C75" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D75" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E75" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F75" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G75" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H75" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I75" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J75" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K75" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L75" s="6" t="n">
-        <v>0.8727</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="3" t="n">
-        <v>1884</v>
-      </c>
-      <c r="B76" s="3" t="n">
-        <v>2337</v>
-      </c>
-      <c r="C76" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D76" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E76" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F76" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G76" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H76" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I76" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J76" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K76" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L76" s="6" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="3" t="n">
-        <v>2337</v>
-      </c>
-      <c r="B77" s="3" t="n">
-        <v>2655</v>
-      </c>
-      <c r="C77" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D77" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E77" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F77" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G77" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H77" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I77" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J77" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K77" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L77" s="6" t="n">
-        <v>0.8727</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="3" t="n">
-        <v>2655</v>
-      </c>
-      <c r="B78" s="3" t="n">
-        <v>2999</v>
-      </c>
-      <c r="C78" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D78" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E78" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F78" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G78" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H78" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I78" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J78" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K78" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L78" s="6" t="n">
-        <v>0.8727</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="n">
-        <v>258</v>
-      </c>
-      <c r="D79" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="E79" s="3" t="n">
-        <v>281</v>
-      </c>
-      <c r="F79" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G79" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H79" s="4" t="n">
-        <v>0.08185053380782918</v>
-      </c>
-      <c r="I79" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J79" s="6" t="n">
-        <v>2.414</v>
-      </c>
-      <c r="K79" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L79" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="1" t="inlineStr">
-        <is>
-          <t>rat1_sum_bu_1_14_pboc_aj65_cur</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>goods</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>bads</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>good_prop</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>bad_prop</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>bad_rate</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>woe</t>
-        </is>
-      </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>iv</t>
-        </is>
-      </c>
-      <c r="K82" s="2" t="inlineStr">
-        <is>
-          <t>ks</t>
-        </is>
-      </c>
-      <c r="L82" s="2" t="inlineStr">
-        <is>
-          <t>lift</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="3" t="n">
-        <v>-999999.001</v>
-      </c>
-      <c r="B83" s="3" t="n">
-        <v>0.0803</v>
-      </c>
-      <c r="C83" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D83" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E83" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="F83" s="5" t="n">
-        <v>0.09302325581395349</v>
-      </c>
-      <c r="G83" s="5" t="n">
-        <v>0.2173913043478261</v>
-      </c>
-      <c r="H83" s="4" t="n">
-        <v>0.1724</v>
-      </c>
-      <c r="I83" s="6" t="n">
-        <v>0.8488</v>
-      </c>
-      <c r="J83" s="6" t="n">
-        <v>0.1056</v>
-      </c>
-      <c r="K83" s="6" t="n">
-        <v>0.1244</v>
-      </c>
-      <c r="L83" s="6" t="n">
-        <v>2.1064</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="3" t="n">
-        <v>0.0803</v>
-      </c>
-      <c r="B84" s="3" t="n">
-        <v>0.258</v>
-      </c>
-      <c r="C84" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D84" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E84" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F84" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G84" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H84" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I84" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J84" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K84" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L84" s="6" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="3" t="n">
-        <v>0.258</v>
-      </c>
-      <c r="B85" s="3" t="n">
-        <v>0.471</v>
-      </c>
-      <c r="C85" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D85" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E85" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F85" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G85" s="5" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H85" s="4" t="n">
-        <v>0.0357</v>
-      </c>
-      <c r="I85" s="6" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J85" s="6" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K85" s="6" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L85" s="6" t="n">
-        <v>0.4363</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="3" t="n">
-        <v>0.471</v>
-      </c>
-      <c r="B86" s="3" t="n">
-        <v>0.669</v>
-      </c>
-      <c r="C86" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D86" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E86" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F86" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G86" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H86" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I86" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J86" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K86" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L86" s="6" t="n">
-        <v>0.8727</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="3" t="n">
-        <v>0.669</v>
-      </c>
-      <c r="B87" s="3" t="n">
-        <v>0.907</v>
-      </c>
-      <c r="C87" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D87" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E87" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F87" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G87" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H87" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I87" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J87" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K87" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L87" s="6" t="n">
-        <v>0.8727</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="3" t="n">
-        <v>0.907</v>
-      </c>
-      <c r="B88" s="3" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="C88" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D88" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E88" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F88" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G88" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H88" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I88" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J88" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K88" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L88" s="6" t="n">
-        <v>0.8727</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="3" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="B89" s="3" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="C89" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D89" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E89" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F89" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G89" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H89" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I89" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J89" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K89" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L89" s="6" t="n">
-        <v>0.8727</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="3" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="B90" s="3" t="n">
-        <v>1.561</v>
-      </c>
-      <c r="C90" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="D90" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E90" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F90" s="5" t="n">
-        <v>0.1007751937984496</v>
-      </c>
-      <c r="G90" s="5" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="H90" s="4" t="n">
-        <v>0.07140000000000001</v>
-      </c>
-      <c r="I90" s="6" t="n">
-        <v>-0.1475</v>
-      </c>
-      <c r="J90" s="6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K90" s="6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="L90" s="6" t="n">
-        <v>0.8727</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="3" t="n">
-        <v>1.561</v>
-      </c>
-      <c r="B91" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="C91" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="D91" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E91" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F91" s="5" t="n">
-        <v>0.09689922480620156</v>
-      </c>
-      <c r="G91" s="5" t="n">
-        <v>0.1304347826086956</v>
-      </c>
-      <c r="H91" s="4" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="I91" s="6" t="n">
-        <v>0.2972</v>
-      </c>
-      <c r="J91" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K91" s="6" t="n">
-        <v>0.0335</v>
-      </c>
-      <c r="L91" s="6" t="n">
-        <v>1.309</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="B92" s="3" t="n">
-        <v>1.996</v>
-      </c>
-      <c r="C92" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D92" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E92" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="F92" s="5" t="n">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="G92" s="5" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H92" s="4" t="n">
-        <v>0.0357</v>
-      </c>
-      <c r="I92" s="6" t="n">
-        <v>-0.8784</v>
-      </c>
-      <c r="J92" s="6" t="n">
-        <v>0.0537</v>
-      </c>
-      <c r="K92" s="6" t="n">
-        <v>0.0612</v>
-      </c>
-      <c r="L92" s="6" t="n">
-        <v>0.4363</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C93" s="3" t="n">
-        <v>258</v>
-      </c>
-      <c r="D93" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="E93" s="3" t="n">
-        <v>281</v>
-      </c>
-      <c r="F93" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G93" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H93" s="4" t="n">
-        <v>0.08185053380782918</v>
-      </c>
-      <c r="I93" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J93" s="6" t="n">
-        <v>0.243</v>
-      </c>
-      <c r="K93" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L93" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="1" t="inlineStr">
-        <is>
-          <t>r24m_cfcbnkndpst_noacct_ln_tac</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>goods</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>bads</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="F96" s="2" t="inlineStr">
-        <is>
-          <t>good_prop</t>
-        </is>
-      </c>
-      <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t>bad_prop</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr">
-        <is>
-          <t>bad_rate</t>
-        </is>
-      </c>
-      <c r="I96" s="2" t="inlineStr">
-        <is>
-          <t>woe</t>
-        </is>
-      </c>
-      <c r="J96" s="2" t="inlineStr">
-        <is>
-          <t>iv</t>
-        </is>
-      </c>
-      <c r="K96" s="2" t="inlineStr">
-        <is>
-          <t>ks</t>
-        </is>
-      </c>
-      <c r="L96" s="2" t="inlineStr">
-        <is>
-          <t>lift</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="3" t="n">
-        <v>-0.001</v>
-      </c>
-      <c r="B97" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C97" s="3" t="n">
-        <v>185</v>
-      </c>
-      <c r="D97" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="E97" s="3" t="n">
-        <v>199</v>
-      </c>
-      <c r="F97" s="5" t="n">
-        <v>0.7170542635658915</v>
-      </c>
-      <c r="G97" s="5" t="n">
-        <v>0.6086956521739131</v>
-      </c>
-      <c r="H97" s="4" t="n">
-        <v>0.0704</v>
-      </c>
-      <c r="I97" s="6" t="n">
-        <v>-0.1638</v>
-      </c>
-      <c r="J97" s="6" t="n">
-        <v>0.0178</v>
-      </c>
-      <c r="K97" s="6" t="n">
-        <v>0.1084</v>
-      </c>
-      <c r="L97" s="6" t="n">
-        <v>0.8595</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B98" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C98" s="3" t="n">
-        <v>73</v>
-      </c>
-      <c r="D98" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="E98" s="3" t="n">
-        <v>82</v>
-      </c>
-      <c r="F98" s="5" t="n">
-        <v>0.2829457364341085</v>
-      </c>
-      <c r="G98" s="5" t="n">
-        <v>0.391304347826087</v>
-      </c>
-      <c r="H98" s="4" t="n">
-        <v>0.1098</v>
-      </c>
-      <c r="I98" s="6" t="n">
-        <v>0.3242</v>
-      </c>
-      <c r="J98" s="6" t="n">
-        <v>0.0351</v>
-      </c>
-      <c r="K98" s="6" t="n">
-        <v>0.1084</v>
-      </c>
-      <c r="L98" s="6" t="n">
-        <v>1.3409</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B99" s="3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="C99" s="3" t="n">
-        <v>258</v>
-      </c>
-      <c r="D99" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="E99" s="3" t="n">
-        <v>281</v>
-      </c>
-      <c r="F99" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G99" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H99" s="4" t="n">
-        <v>0.08185053380782918</v>
-      </c>
-      <c r="I99" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J99" s="6" t="n">
-        <v>0.0529</v>
-      </c>
-      <c r="K99" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L99" s="6" t="n">
-        <v>1</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H13:H23">
+  <conditionalFormatting sqref="H13:H15">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4657,7 +3209,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I13:I23">
+  <conditionalFormatting sqref="I13:I15">
     <cfRule type="dataBar" priority="2">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4666,7 +3218,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L13:L23">
+  <conditionalFormatting sqref="L13:L15">
     <cfRule type="dataBar" priority="3">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4675,7 +3227,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H27:H37">
+  <conditionalFormatting sqref="H19:H24">
     <cfRule type="dataBar" priority="4">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4684,7 +3236,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I27:I37">
+  <conditionalFormatting sqref="I19:I24">
     <cfRule type="dataBar" priority="5">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4693,7 +3245,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L27:L37">
+  <conditionalFormatting sqref="L19:L24">
     <cfRule type="dataBar" priority="6">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4702,7 +3254,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H41:H51">
+  <conditionalFormatting sqref="H28:H30">
     <cfRule type="dataBar" priority="7">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4711,7 +3263,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I41:I51">
+  <conditionalFormatting sqref="I28:I30">
     <cfRule type="dataBar" priority="8">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4720,7 +3272,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L41:L51">
+  <conditionalFormatting sqref="L28:L30">
     <cfRule type="dataBar" priority="9">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4729,7 +3281,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H55:H65">
+  <conditionalFormatting sqref="H34:H38">
     <cfRule type="dataBar" priority="10">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4738,7 +3290,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I55:I65">
+  <conditionalFormatting sqref="I34:I38">
     <cfRule type="dataBar" priority="11">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4747,7 +3299,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L55:L65">
+  <conditionalFormatting sqref="L34:L38">
     <cfRule type="dataBar" priority="12">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4756,7 +3308,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H69:H79">
+  <conditionalFormatting sqref="H42:H47">
     <cfRule type="dataBar" priority="13">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4765,7 +3317,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I69:I79">
+  <conditionalFormatting sqref="I42:I47">
     <cfRule type="dataBar" priority="14">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4774,7 +3326,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L69:L79">
+  <conditionalFormatting sqref="L42:L47">
     <cfRule type="dataBar" priority="15">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4783,7 +3335,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H83:H93">
+  <conditionalFormatting sqref="H51:H54">
     <cfRule type="dataBar" priority="16">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4792,7 +3344,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I83:I93">
+  <conditionalFormatting sqref="I51:I54">
     <cfRule type="dataBar" priority="17">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4801,7 +3353,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L83:L93">
+  <conditionalFormatting sqref="L51:L54">
     <cfRule type="dataBar" priority="18">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4810,7 +3362,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H97:H99">
+  <conditionalFormatting sqref="H58:H60">
     <cfRule type="dataBar" priority="19">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4819,7 +3371,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I97:I99">
+  <conditionalFormatting sqref="I58:I60">
     <cfRule type="dataBar" priority="20">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -4828,7 +3380,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L97:L99">
+  <conditionalFormatting sqref="L58:L60">
     <cfRule type="dataBar" priority="21">
       <dataBar showValue="1">
         <cfvo type="min"/>

</xml_diff>

<commit_message>
fix: data bars minLength=5 for visibility at zero values
</commit_message>
<xml_diff>
--- a/sample_report.xlsx
+++ b/sample_report.xlsx
@@ -3202,7 +3202,7 @@
   </sheetData>
   <conditionalFormatting sqref="H13:H15">
     <cfRule type="dataBar" priority="1">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3211,7 +3211,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="I13:I15">
     <cfRule type="dataBar" priority="2">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3220,7 +3220,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L13:L15">
     <cfRule type="dataBar" priority="3">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3229,7 +3229,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H19:H24">
     <cfRule type="dataBar" priority="4">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3238,7 +3238,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="I19:I24">
     <cfRule type="dataBar" priority="5">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3247,7 +3247,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L19:L24">
     <cfRule type="dataBar" priority="6">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3256,7 +3256,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H28:H30">
     <cfRule type="dataBar" priority="7">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3265,7 +3265,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="I28:I30">
     <cfRule type="dataBar" priority="8">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3274,7 +3274,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L28:L30">
     <cfRule type="dataBar" priority="9">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3283,7 +3283,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H34:H38">
     <cfRule type="dataBar" priority="10">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3292,7 +3292,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="I34:I38">
     <cfRule type="dataBar" priority="11">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3301,7 +3301,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L34:L38">
     <cfRule type="dataBar" priority="12">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3310,7 +3310,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H42:H47">
     <cfRule type="dataBar" priority="13">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3319,7 +3319,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="I42:I47">
     <cfRule type="dataBar" priority="14">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3328,7 +3328,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L42:L47">
     <cfRule type="dataBar" priority="15">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3337,7 +3337,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H51:H54">
     <cfRule type="dataBar" priority="16">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3346,7 +3346,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="I51:I54">
     <cfRule type="dataBar" priority="17">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3355,7 +3355,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L51:L54">
     <cfRule type="dataBar" priority="18">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3364,7 +3364,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H58:H60">
     <cfRule type="dataBar" priority="19">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3373,7 +3373,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="I58:I60">
     <cfRule type="dataBar" priority="20">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -3382,7 +3382,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L58:L60">
     <cfRule type="dataBar" priority="21">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9811,7 +9811,7 @@
   </sheetData>
   <conditionalFormatting sqref="J14:J16">
     <cfRule type="dataBar" priority="1">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9820,7 +9820,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K14:K16">
     <cfRule type="dataBar" priority="2">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9829,7 +9829,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L14:L16">
     <cfRule type="dataBar" priority="3">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9838,7 +9838,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="M14:M16">
     <cfRule type="dataBar" priority="4">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9847,7 +9847,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L20:L29">
     <cfRule type="dataBar" priority="5">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9856,7 +9856,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="M20:M29">
     <cfRule type="dataBar" priority="6">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9865,7 +9865,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="N20:N29">
     <cfRule type="dataBar" priority="7">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9874,7 +9874,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="O20:O29">
     <cfRule type="dataBar" priority="8">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9883,7 +9883,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F33:F42">
     <cfRule type="dataBar" priority="9">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9892,7 +9892,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G33:G42">
     <cfRule type="dataBar" priority="10">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9901,7 +9901,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J33:J42">
     <cfRule type="dataBar" priority="11">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9910,7 +9910,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K33:K42">
     <cfRule type="dataBar" priority="12">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9919,7 +9919,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F46:F55">
     <cfRule type="dataBar" priority="13">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9928,7 +9928,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G46:G55">
     <cfRule type="dataBar" priority="14">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9937,7 +9937,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J46:J55">
     <cfRule type="dataBar" priority="15">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9946,7 +9946,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K46:K55">
     <cfRule type="dataBar" priority="16">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9955,7 +9955,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F59:F68">
     <cfRule type="dataBar" priority="17">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9964,7 +9964,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G59:G68">
     <cfRule type="dataBar" priority="18">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9973,7 +9973,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J59:J68">
     <cfRule type="dataBar" priority="19">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9982,7 +9982,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K59:K68">
     <cfRule type="dataBar" priority="20">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -9991,7 +9991,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F72:F81">
     <cfRule type="dataBar" priority="21">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10000,7 +10000,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G72:G81">
     <cfRule type="dataBar" priority="22">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10009,7 +10009,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J72:J81">
     <cfRule type="dataBar" priority="23">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10018,7 +10018,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K72:K81">
     <cfRule type="dataBar" priority="24">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10027,7 +10027,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F85:F94">
     <cfRule type="dataBar" priority="25">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10036,7 +10036,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G85:G94">
     <cfRule type="dataBar" priority="26">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10045,7 +10045,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J85:J94">
     <cfRule type="dataBar" priority="27">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10054,7 +10054,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K85:K94">
     <cfRule type="dataBar" priority="28">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10063,7 +10063,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F107">
     <cfRule type="dataBar" priority="29">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10072,7 +10072,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G98:G107">
     <cfRule type="dataBar" priority="30">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10081,7 +10081,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J98:J107">
     <cfRule type="dataBar" priority="31">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10090,7 +10090,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K98:K107">
     <cfRule type="dataBar" priority="32">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10099,7 +10099,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F111:F120">
     <cfRule type="dataBar" priority="33">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10108,7 +10108,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G111:G120">
     <cfRule type="dataBar" priority="34">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10117,7 +10117,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J111:J120">
     <cfRule type="dataBar" priority="35">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10126,7 +10126,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K111:K120">
     <cfRule type="dataBar" priority="36">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10135,7 +10135,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F124:F133">
     <cfRule type="dataBar" priority="37">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10144,7 +10144,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G124:G133">
     <cfRule type="dataBar" priority="38">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10153,7 +10153,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J124:J133">
     <cfRule type="dataBar" priority="39">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10162,7 +10162,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K124:K133">
     <cfRule type="dataBar" priority="40">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10171,7 +10171,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F137:F146">
     <cfRule type="dataBar" priority="41">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10180,7 +10180,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G137:G146">
     <cfRule type="dataBar" priority="42">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10189,7 +10189,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J137:J146">
     <cfRule type="dataBar" priority="43">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10198,7 +10198,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K137:K146">
     <cfRule type="dataBar" priority="44">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10207,7 +10207,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F150:F159">
     <cfRule type="dataBar" priority="45">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10216,7 +10216,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G150:G159">
     <cfRule type="dataBar" priority="46">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10225,7 +10225,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J150:J159">
     <cfRule type="dataBar" priority="47">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10234,7 +10234,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K150:K159">
     <cfRule type="dataBar" priority="48">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10243,7 +10243,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F163:F172">
     <cfRule type="dataBar" priority="49">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10252,7 +10252,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G163:G172">
     <cfRule type="dataBar" priority="50">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10261,7 +10261,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J163:J172">
     <cfRule type="dataBar" priority="51">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10270,7 +10270,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K163:K172">
     <cfRule type="dataBar" priority="52">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10279,7 +10279,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F176:F185">
     <cfRule type="dataBar" priority="53">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10288,7 +10288,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G176:G185">
     <cfRule type="dataBar" priority="54">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10297,7 +10297,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J176:J185">
     <cfRule type="dataBar" priority="55">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>
@@ -10306,7 +10306,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K176:K185">
     <cfRule type="dataBar" priority="56">
-      <dataBar showValue="1">
+      <dataBar minLength="5" maxLength="100" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FF5B9BD5"/>

</xml_diff>

<commit_message>
format: bin_performance bad_rate/cum_bad_rate/cum_bads_prop as 0.00%
- bad_rate: 0.0000 → 0.00% (percentage, 2dp)
- cum_bad_rate: 0.0000 → 0.00%
- cum_bads_prop: 0.0000 → 0.00%
- ks/lift/cum_lift: already 0.00 (unchanged)
- Applies to both Sheet 2 WOE tables and Sheet 3 bin performance
</commit_message>
<xml_diff>
--- a/sample_report.xlsx
+++ b/sample_report.xlsx
@@ -1607,7 +1607,7 @@
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="H13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="6" t="n">
@@ -1647,7 +1647,7 @@
       <c r="G14" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="H14" s="5" t="n">
         <v>0.0895</v>
       </c>
       <c r="I14" s="6" t="n">
@@ -1689,7 +1689,7 @@
       <c r="G15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="H15" s="5" t="n">
         <v>0.08185053380782918</v>
       </c>
       <c r="I15" s="6" t="n">
@@ -1798,7 +1798,7 @@
       <c r="G19" s="5" t="n">
         <v>0.3043478260869565</v>
       </c>
-      <c r="H19" s="4" t="n">
+      <c r="H19" s="5" t="n">
         <v>0.0625</v>
       </c>
       <c r="I19" s="6" t="n">
@@ -1836,7 +1836,7 @@
       <c r="G20" s="5" t="n">
         <v>0.3043478260869565</v>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="H20" s="5" t="n">
         <v>0.0625</v>
       </c>
       <c r="I20" s="6" t="n">
@@ -1874,7 +1874,7 @@
       <c r="G21" s="5" t="n">
         <v>0.04347826086956522</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="H21" s="5" t="n">
         <v>0.07140000000000001</v>
       </c>
       <c r="I21" s="6" t="n">
@@ -1912,7 +1912,7 @@
       <c r="G22" s="5" t="n">
         <v>0.08695652173913043</v>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="H22" s="5" t="n">
         <v>0.1429</v>
       </c>
       <c r="I22" s="6" t="n">
@@ -1952,7 +1952,7 @@
       <c r="G23" s="5" t="n">
         <v>0.2608695652173913</v>
       </c>
-      <c r="H23" s="4" t="n">
+      <c r="H23" s="5" t="n">
         <v>0.2069</v>
       </c>
       <c r="I23" s="6" t="n">
@@ -1994,7 +1994,7 @@
       <c r="G24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H24" s="4" t="n">
+      <c r="H24" s="5" t="n">
         <v>0.08185053380782918</v>
       </c>
       <c r="I24" s="6" t="n">
@@ -2103,7 +2103,7 @@
       <c r="G28" s="5" t="n">
         <v>0.7826086956521739</v>
       </c>
-      <c r="H28" s="4" t="n">
+      <c r="H28" s="5" t="n">
         <v>0.0756</v>
       </c>
       <c r="I28" s="6" t="n">
@@ -2143,7 +2143,7 @@
       <c r="G29" s="5" t="n">
         <v>0.2173913043478261</v>
       </c>
-      <c r="H29" s="4" t="n">
+      <c r="H29" s="5" t="n">
         <v>0.1163</v>
       </c>
       <c r="I29" s="6" t="n">
@@ -2185,7 +2185,7 @@
       <c r="G30" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H30" s="4" t="n">
+      <c r="H30" s="5" t="n">
         <v>0.08185053380782918</v>
       </c>
       <c r="I30" s="6" t="n">
@@ -2294,7 +2294,7 @@
       <c r="G34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="4" t="n">
+      <c r="H34" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I34" s="6" t="n">
@@ -2332,7 +2332,7 @@
       <c r="G35" s="5" t="n">
         <v>0.6956521739130435</v>
       </c>
-      <c r="H35" s="4" t="n">
+      <c r="H35" s="5" t="n">
         <v>0.0762</v>
       </c>
       <c r="I35" s="6" t="n">
@@ -2370,7 +2370,7 @@
       <c r="G36" s="5" t="n">
         <v>0.1739130434782609</v>
       </c>
-      <c r="H36" s="4" t="n">
+      <c r="H36" s="5" t="n">
         <v>0.09520000000000001</v>
       </c>
       <c r="I36" s="6" t="n">
@@ -2410,7 +2410,7 @@
       <c r="G37" s="5" t="n">
         <v>0.1304347826086956</v>
       </c>
-      <c r="H37" s="4" t="n">
+      <c r="H37" s="5" t="n">
         <v>0.2</v>
       </c>
       <c r="I37" s="6" t="n">
@@ -2452,7 +2452,7 @@
       <c r="G38" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H38" s="4" t="n">
+      <c r="H38" s="5" t="n">
         <v>0.08185053380782918</v>
       </c>
       <c r="I38" s="6" t="n">
@@ -2563,7 +2563,7 @@
       <c r="G42" s="5" t="n">
         <v>0.04347826086956522</v>
       </c>
-      <c r="H42" s="4" t="n">
+      <c r="H42" s="5" t="n">
         <v>0.07140000000000001</v>
       </c>
       <c r="I42" s="6" t="n">
@@ -2603,7 +2603,7 @@
       <c r="G43" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="4" t="n">
+      <c r="H43" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I43" s="6" t="n">
@@ -2641,7 +2641,7 @@
       <c r="G44" s="5" t="n">
         <v>0.04347826086956522</v>
       </c>
-      <c r="H44" s="4" t="n">
+      <c r="H44" s="5" t="n">
         <v>0.0769</v>
       </c>
       <c r="I44" s="6" t="n">
@@ -2679,7 +2679,7 @@
       <c r="G45" s="5" t="n">
         <v>0.6086956521739131</v>
       </c>
-      <c r="H45" s="4" t="n">
+      <c r="H45" s="5" t="n">
         <v>0.08749999999999999</v>
       </c>
       <c r="I45" s="6" t="n">
@@ -2719,7 +2719,7 @@
       <c r="G46" s="5" t="n">
         <v>0.3043478260869565</v>
       </c>
-      <c r="H46" s="4" t="n">
+      <c r="H46" s="5" t="n">
         <v>0.08749999999999999</v>
       </c>
       <c r="I46" s="6" t="n">
@@ -2761,7 +2761,7 @@
       <c r="G47" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H47" s="4" t="n">
+      <c r="H47" s="5" t="n">
         <v>0.08185053380782918</v>
       </c>
       <c r="I47" s="6" t="n">
@@ -2872,7 +2872,7 @@
       <c r="G51" s="5" t="n">
         <v>0.08695652173913043</v>
       </c>
-      <c r="H51" s="4" t="n">
+      <c r="H51" s="5" t="n">
         <v>0.1176</v>
       </c>
       <c r="I51" s="6" t="n">
@@ -2912,7 +2912,7 @@
       <c r="G52" s="5" t="n">
         <v>0.6521739130434783</v>
       </c>
-      <c r="H52" s="4" t="n">
+      <c r="H52" s="5" t="n">
         <v>0.07580000000000001</v>
       </c>
       <c r="I52" s="6" t="n">
@@ -2952,7 +2952,7 @@
       <c r="G53" s="5" t="n">
         <v>0.2608695652173913</v>
       </c>
-      <c r="H53" s="4" t="n">
+      <c r="H53" s="5" t="n">
         <v>0.09089999999999999</v>
       </c>
       <c r="I53" s="6" t="n">
@@ -2994,7 +2994,7 @@
       <c r="G54" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H54" s="4" t="n">
+      <c r="H54" s="5" t="n">
         <v>0.08185053380782918</v>
       </c>
       <c r="I54" s="6" t="n">
@@ -3101,7 +3101,7 @@
       <c r="G58" s="5" t="n">
         <v>0.6086956521739131</v>
       </c>
-      <c r="H58" s="4" t="n">
+      <c r="H58" s="5" t="n">
         <v>0.0704</v>
       </c>
       <c r="I58" s="6" t="n">
@@ -3141,7 +3141,7 @@
       <c r="G59" s="5" t="n">
         <v>0.391304347826087</v>
       </c>
-      <c r="H59" s="4" t="n">
+      <c r="H59" s="5" t="n">
         <v>0.1098</v>
       </c>
       <c r="I59" s="6" t="n">
@@ -3183,7 +3183,7 @@
       <c r="G60" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H60" s="4" t="n">
+      <c r="H60" s="5" t="n">
         <v>0.08185053380782918</v>
       </c>
       <c r="I60" s="6" t="n">
@@ -4874,13 +4874,13 @@
       <c r="E33" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="F33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="4" t="n">
+      <c r="F33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="6" t="n">
@@ -4909,13 +4909,13 @@
       <c r="E34" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="F34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="4" t="n">
+      <c r="F34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I34" s="6" t="n">
@@ -4944,13 +4944,13 @@
       <c r="E35" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="F35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="4" t="n">
+      <c r="F35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="6" t="n">
@@ -4979,13 +4979,13 @@
       <c r="E36" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="F36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="4" t="n">
+      <c r="F36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I36" s="6" t="n">
@@ -5014,13 +5014,13 @@
       <c r="E37" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="F37" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="4" t="n">
+      <c r="F37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I37" s="6" t="n">
@@ -5049,13 +5049,13 @@
       <c r="E38" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="F38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="4" t="n">
+      <c r="F38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I38" s="6" t="n">
@@ -5084,13 +5084,13 @@
       <c r="E39" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="F39" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="4" t="n">
+      <c r="F39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="6" t="n">
@@ -5119,13 +5119,13 @@
       <c r="E40" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="F40" s="4" t="n">
+      <c r="F40" s="5" t="n">
         <v>0.0357</v>
       </c>
-      <c r="G40" s="4" t="n">
+      <c r="G40" s="5" t="n">
         <v>0.0044</v>
       </c>
-      <c r="H40" s="4" t="n">
+      <c r="H40" s="5" t="n">
         <v>0.0435</v>
       </c>
       <c r="I40" s="6" t="n">
@@ -5154,13 +5154,13 @@
       <c r="E41" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="F41" s="4" t="n">
+      <c r="F41" s="5" t="n">
         <v>0.25</v>
       </c>
-      <c r="G41" s="4" t="n">
+      <c r="G41" s="5" t="n">
         <v>0.0316</v>
       </c>
-      <c r="H41" s="4" t="n">
+      <c r="H41" s="5" t="n">
         <v>0.3478</v>
       </c>
       <c r="I41" s="6" t="n">
@@ -5191,13 +5191,13 @@
       <c r="E42" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="F42" s="4" t="n">
+      <c r="F42" s="5" t="n">
         <v>0.5357</v>
       </c>
-      <c r="G42" s="4" t="n">
+      <c r="G42" s="5" t="n">
         <v>0.0819</v>
       </c>
-      <c r="H42" s="4" t="n">
+      <c r="H42" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I42" s="6" t="n">
@@ -5292,13 +5292,13 @@
       <c r="E46" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="4" t="n">
+      <c r="F46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I46" s="6" t="n">
@@ -5327,13 +5327,13 @@
       <c r="E47" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="4" t="n">
+      <c r="F47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I47" s="6" t="n">
@@ -5362,13 +5362,13 @@
       <c r="E48" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F48" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="4" t="n">
+      <c r="F48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I48" s="6" t="n">
@@ -5397,13 +5397,13 @@
       <c r="E49" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F49" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="4" t="n">
+      <c r="F49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I49" s="6" t="n">
@@ -5432,13 +5432,13 @@
       <c r="E50" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F50" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="4" t="n">
+      <c r="F50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I50" s="6" t="n">
@@ -5467,13 +5467,13 @@
       <c r="E51" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F51" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="4" t="n">
+      <c r="F51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I51" s="6" t="n">
@@ -5502,13 +5502,13 @@
       <c r="E52" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F52" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G52" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H52" s="4" t="n">
+      <c r="F52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I52" s="6" t="n">
@@ -5537,13 +5537,13 @@
       <c r="E53" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F53" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="4" t="n">
+      <c r="F53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I53" s="6" t="n">
@@ -5572,13 +5572,13 @@
       <c r="E54" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F54" s="4" t="n">
+      <c r="F54" s="5" t="n">
         <v>0.25</v>
       </c>
-      <c r="G54" s="4" t="n">
+      <c r="G54" s="5" t="n">
         <v>0.0282</v>
       </c>
-      <c r="H54" s="4" t="n">
+      <c r="H54" s="5" t="n">
         <v>0.5</v>
       </c>
       <c r="I54" s="6" t="n">
@@ -5609,13 +5609,13 @@
       <c r="E55" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F55" s="4" t="n">
+      <c r="F55" s="5" t="n">
         <v>0.25</v>
       </c>
-      <c r="G55" s="4" t="n">
+      <c r="G55" s="5" t="n">
         <v>0.0506</v>
       </c>
-      <c r="H55" s="4" t="n">
+      <c r="H55" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I55" s="6" t="n">
@@ -5710,13 +5710,13 @@
       <c r="E59" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F59" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="4" t="n">
+      <c r="F59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I59" s="6" t="n">
@@ -5745,13 +5745,13 @@
       <c r="E60" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F60" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="4" t="n">
+      <c r="F60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I60" s="6" t="n">
@@ -5780,13 +5780,13 @@
       <c r="E61" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F61" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H61" s="4" t="n">
+      <c r="F61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I61" s="6" t="n">
@@ -5815,13 +5815,13 @@
       <c r="E62" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F62" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G62" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H62" s="4" t="n">
+      <c r="F62" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I62" s="6" t="n">
@@ -5850,13 +5850,13 @@
       <c r="E63" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F63" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G63" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H63" s="4" t="n">
+      <c r="F63" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I63" s="6" t="n">
@@ -5885,13 +5885,13 @@
       <c r="E64" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F64" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G64" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H64" s="4" t="n">
+      <c r="F64" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I64" s="6" t="n">
@@ -5920,13 +5920,13 @@
       <c r="E65" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F65" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G65" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" s="4" t="n">
+      <c r="F65" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I65" s="6" t="n">
@@ -5955,13 +5955,13 @@
       <c r="E66" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F66" s="4" t="n">
+      <c r="F66" s="5" t="n">
         <v>0.1</v>
       </c>
-      <c r="G66" s="4" t="n">
+      <c r="G66" s="5" t="n">
         <v>0.0125</v>
       </c>
-      <c r="H66" s="4" t="n">
+      <c r="H66" s="5" t="n">
         <v>0.125</v>
       </c>
       <c r="I66" s="6" t="n">
@@ -5990,13 +5990,13 @@
       <c r="E67" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F67" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G67" s="4" t="n">
+      <c r="F67" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="5" t="n">
         <v>0.0111</v>
       </c>
-      <c r="H67" s="4" t="n">
+      <c r="H67" s="5" t="n">
         <v>0.125</v>
       </c>
       <c r="I67" s="6" t="n">
@@ -6027,13 +6027,13 @@
       <c r="E68" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F68" s="4" t="n">
+      <c r="F68" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="G68" s="4" t="n">
+      <c r="G68" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="H68" s="4" t="n">
+      <c r="H68" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I68" s="6" t="n">
@@ -6128,13 +6128,13 @@
       <c r="E72" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F72" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G72" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H72" s="4" t="n">
+      <c r="F72" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I72" s="6" t="n">
@@ -6163,13 +6163,13 @@
       <c r="E73" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F73" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H73" s="4" t="n">
+      <c r="F73" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I73" s="6" t="n">
@@ -6198,13 +6198,13 @@
       <c r="E74" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F74" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G74" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H74" s="4" t="n">
+      <c r="F74" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I74" s="6" t="n">
@@ -6233,13 +6233,13 @@
       <c r="E75" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F75" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G75" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H75" s="4" t="n">
+      <c r="F75" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I75" s="6" t="n">
@@ -6268,13 +6268,13 @@
       <c r="E76" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F76" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G76" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H76" s="4" t="n">
+      <c r="F76" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I76" s="6" t="n">
@@ -6303,13 +6303,13 @@
       <c r="E77" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F77" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G77" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H77" s="4" t="n">
+      <c r="F77" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I77" s="6" t="n">
@@ -6338,13 +6338,13 @@
       <c r="E78" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F78" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G78" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H78" s="4" t="n">
+      <c r="F78" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I78" s="6" t="n">
@@ -6373,13 +6373,13 @@
       <c r="E79" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F79" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G79" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H79" s="4" t="n">
+      <c r="F79" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I79" s="6" t="n">
@@ -6408,13 +6408,13 @@
       <c r="E80" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F80" s="4" t="n">
+      <c r="F80" s="5" t="n">
         <v>0.1667</v>
       </c>
-      <c r="G80" s="4" t="n">
+      <c r="G80" s="5" t="n">
         <v>0.0185</v>
       </c>
-      <c r="H80" s="4" t="n">
+      <c r="H80" s="5" t="n">
         <v>0.2</v>
       </c>
       <c r="I80" s="6" t="n">
@@ -6445,13 +6445,13 @@
       <c r="E81" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F81" s="4" t="n">
+      <c r="F81" s="5" t="n">
         <v>0.6667</v>
       </c>
-      <c r="G81" s="4" t="n">
+      <c r="G81" s="5" t="n">
         <v>0.0833</v>
       </c>
-      <c r="H81" s="4" t="n">
+      <c r="H81" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I81" s="6" t="n">
@@ -6546,13 +6546,13 @@
       <c r="E85" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F85" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G85" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H85" s="4" t="n">
+      <c r="F85" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I85" s="6" t="n">
@@ -6581,13 +6581,13 @@
       <c r="E86" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F86" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G86" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H86" s="4" t="n">
+      <c r="F86" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I86" s="6" t="n">
@@ -6616,13 +6616,13 @@
       <c r="E87" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F87" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G87" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H87" s="4" t="n">
+      <c r="F87" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I87" s="6" t="n">
@@ -6651,13 +6651,13 @@
       <c r="E88" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F88" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G88" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H88" s="4" t="n">
+      <c r="F88" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I88" s="6" t="n">
@@ -6686,13 +6686,13 @@
       <c r="E89" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F89" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G89" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H89" s="4" t="n">
+      <c r="F89" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I89" s="6" t="n">
@@ -6721,13 +6721,13 @@
       <c r="E90" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F90" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G90" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H90" s="4" t="n">
+      <c r="F90" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I90" s="6" t="n">
@@ -6756,13 +6756,13 @@
       <c r="E91" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F91" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G91" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H91" s="4" t="n">
+      <c r="F91" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I91" s="6" t="n">
@@ -6791,13 +6791,13 @@
       <c r="E92" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F92" s="4" t="n">
+      <c r="F92" s="5" t="n">
         <v>0.1667</v>
       </c>
-      <c r="G92" s="4" t="n">
+      <c r="G92" s="5" t="n">
         <v>0.0208</v>
       </c>
-      <c r="H92" s="4" t="n">
+      <c r="H92" s="5" t="n">
         <v>0.1429</v>
       </c>
       <c r="I92" s="6" t="n">
@@ -6826,13 +6826,13 @@
       <c r="E93" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F93" s="4" t="n">
+      <c r="F93" s="5" t="n">
         <v>0.1667</v>
       </c>
-      <c r="G93" s="4" t="n">
+      <c r="G93" s="5" t="n">
         <v>0.037</v>
       </c>
-      <c r="H93" s="4" t="n">
+      <c r="H93" s="5" t="n">
         <v>0.2857</v>
       </c>
       <c r="I93" s="6" t="n">
@@ -6863,13 +6863,13 @@
       <c r="E94" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F94" s="4" t="n">
+      <c r="F94" s="5" t="n">
         <v>0.8333</v>
       </c>
-      <c r="G94" s="4" t="n">
+      <c r="G94" s="5" t="n">
         <v>0.1167</v>
       </c>
-      <c r="H94" s="4" t="n">
+      <c r="H94" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I94" s="6" t="n">
@@ -6964,13 +6964,13 @@
       <c r="E98" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F98" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G98" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H98" s="4" t="n">
+      <c r="F98" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I98" s="6" t="n">
@@ -6999,13 +6999,13 @@
       <c r="E99" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F99" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G99" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H99" s="4" t="n">
+      <c r="F99" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I99" s="6" t="n">
@@ -7034,13 +7034,13 @@
       <c r="E100" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F100" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G100" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H100" s="4" t="n">
+      <c r="F100" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I100" s="6" t="n">
@@ -7069,13 +7069,13 @@
       <c r="E101" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F101" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G101" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H101" s="4" t="n">
+      <c r="F101" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I101" s="6" t="n">
@@ -7104,13 +7104,13 @@
       <c r="E102" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F102" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G102" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H102" s="4" t="n">
+      <c r="F102" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I102" s="6" t="n">
@@ -7139,13 +7139,13 @@
       <c r="E103" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F103" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G103" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H103" s="4" t="n">
+      <c r="F103" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I103" s="6" t="n">
@@ -7174,13 +7174,13 @@
       <c r="E104" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F104" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G104" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H104" s="4" t="n">
+      <c r="F104" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I104" s="6" t="n">
@@ -7209,13 +7209,13 @@
       <c r="E105" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F105" s="4" t="n">
+      <c r="F105" s="5" t="n">
         <v>0.1667</v>
       </c>
-      <c r="G105" s="4" t="n">
+      <c r="G105" s="5" t="n">
         <v>0.0208</v>
       </c>
-      <c r="H105" s="4" t="n">
+      <c r="H105" s="5" t="n">
         <v>0.25</v>
       </c>
       <c r="I105" s="6" t="n">
@@ -7244,13 +7244,13 @@
       <c r="E106" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F106" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G106" s="4" t="n">
+      <c r="F106" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" s="5" t="n">
         <v>0.0185</v>
       </c>
-      <c r="H106" s="4" t="n">
+      <c r="H106" s="5" t="n">
         <v>0.25</v>
       </c>
       <c r="I106" s="6" t="n">
@@ -7281,13 +7281,13 @@
       <c r="E107" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F107" s="4" t="n">
+      <c r="F107" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="G107" s="4" t="n">
+      <c r="G107" s="5" t="n">
         <v>0.0667</v>
       </c>
-      <c r="H107" s="4" t="n">
+      <c r="H107" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I107" s="6" t="n">
@@ -7382,13 +7382,13 @@
       <c r="E111" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F111" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G111" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H111" s="4" t="n">
+      <c r="F111" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I111" s="6" t="n">
@@ -7417,13 +7417,13 @@
       <c r="E112" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F112" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G112" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H112" s="4" t="n">
+      <c r="F112" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I112" s="6" t="n">
@@ -7452,13 +7452,13 @@
       <c r="E113" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F113" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G113" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H113" s="4" t="n">
+      <c r="F113" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I113" s="6" t="n">
@@ -7487,13 +7487,13 @@
       <c r="E114" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F114" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G114" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H114" s="4" t="n">
+      <c r="F114" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I114" s="6" t="n">
@@ -7522,13 +7522,13 @@
       <c r="E115" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F115" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G115" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H115" s="4" t="n">
+      <c r="F115" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I115" s="6" t="n">
@@ -7557,13 +7557,13 @@
       <c r="E116" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F116" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G116" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H116" s="4" t="n">
+      <c r="F116" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I116" s="6" t="n">
@@ -7592,13 +7592,13 @@
       <c r="E117" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F117" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G117" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H117" s="4" t="n">
+      <c r="F117" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I117" s="6" t="n">
@@ -7627,13 +7627,13 @@
       <c r="E118" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F118" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G118" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H118" s="4" t="n">
+      <c r="F118" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I118" s="6" t="n">
@@ -7662,13 +7662,13 @@
       <c r="E119" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F119" s="4" t="n">
+      <c r="F119" s="5" t="n">
         <v>0.1667</v>
       </c>
-      <c r="G119" s="4" t="n">
+      <c r="G119" s="5" t="n">
         <v>0.0185</v>
       </c>
-      <c r="H119" s="4" t="n">
+      <c r="H119" s="5" t="n">
         <v>0.5</v>
       </c>
       <c r="I119" s="6" t="n">
@@ -7699,13 +7699,13 @@
       <c r="E120" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F120" s="4" t="n">
+      <c r="F120" s="5" t="n">
         <v>0.1667</v>
       </c>
-      <c r="G120" s="4" t="n">
+      <c r="G120" s="5" t="n">
         <v>0.0333</v>
       </c>
-      <c r="H120" s="4" t="n">
+      <c r="H120" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I120" s="6" t="n">
@@ -7800,13 +7800,13 @@
       <c r="E124" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F124" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G124" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H124" s="4" t="n">
+      <c r="F124" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I124" s="6" t="n">
@@ -7835,13 +7835,13 @@
       <c r="E125" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F125" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G125" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H125" s="4" t="n">
+      <c r="F125" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G125" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I125" s="6" t="n">
@@ -7870,13 +7870,13 @@
       <c r="E126" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F126" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G126" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H126" s="4" t="n">
+      <c r="F126" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G126" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I126" s="6" t="n">
@@ -7905,13 +7905,13 @@
       <c r="E127" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F127" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G127" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H127" s="4" t="n">
+      <c r="F127" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G127" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I127" s="6" t="n">
@@ -7940,13 +7940,13 @@
       <c r="E128" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F128" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G128" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H128" s="4" t="n">
+      <c r="F128" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I128" s="6" t="n">
@@ -7975,13 +7975,13 @@
       <c r="E129" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F129" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G129" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H129" s="4" t="n">
+      <c r="F129" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G129" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I129" s="6" t="n">
@@ -8010,13 +8010,13 @@
       <c r="E130" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F130" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G130" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H130" s="4" t="n">
+      <c r="F130" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I130" s="6" t="n">
@@ -8045,13 +8045,13 @@
       <c r="E131" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F131" s="4" t="n">
+      <c r="F131" s="5" t="n">
         <v>0.1667</v>
       </c>
-      <c r="G131" s="4" t="n">
+      <c r="G131" s="5" t="n">
         <v>0.0208</v>
       </c>
-      <c r="H131" s="4" t="n">
+      <c r="H131" s="5" t="n">
         <v>0.25</v>
       </c>
       <c r="I131" s="6" t="n">
@@ -8080,13 +8080,13 @@
       <c r="E132" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F132" s="4" t="n">
+      <c r="F132" s="5" t="n">
         <v>0.1667</v>
       </c>
-      <c r="G132" s="4" t="n">
+      <c r="G132" s="5" t="n">
         <v>0.037</v>
       </c>
-      <c r="H132" s="4" t="n">
+      <c r="H132" s="5" t="n">
         <v>0.5</v>
       </c>
       <c r="I132" s="6" t="n">
@@ -8117,13 +8117,13 @@
       <c r="E133" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F133" s="4" t="n">
+      <c r="F133" s="5" t="n">
         <v>0.3333</v>
       </c>
-      <c r="G133" s="4" t="n">
+      <c r="G133" s="5" t="n">
         <v>0.0667</v>
       </c>
-      <c r="H133" s="4" t="n">
+      <c r="H133" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I133" s="6" t="n">
@@ -8218,13 +8218,13 @@
       <c r="E137" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F137" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G137" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H137" s="4" t="n">
+      <c r="F137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I137" s="6" t="n">
@@ -8253,13 +8253,13 @@
       <c r="E138" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F138" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G138" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H138" s="4" t="n">
+      <c r="F138" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I138" s="6" t="n">
@@ -8288,13 +8288,13 @@
       <c r="E139" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F139" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G139" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H139" s="4" t="n">
+      <c r="F139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I139" s="6" t="n">
@@ -8323,13 +8323,13 @@
       <c r="E140" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F140" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G140" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H140" s="4" t="n">
+      <c r="F140" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G140" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I140" s="6" t="n">
@@ -8358,13 +8358,13 @@
       <c r="E141" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F141" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G141" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H141" s="4" t="n">
+      <c r="F141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I141" s="6" t="n">
@@ -8393,13 +8393,13 @@
       <c r="E142" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F142" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G142" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H142" s="4" t="n">
+      <c r="F142" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I142" s="6" t="n">
@@ -8428,13 +8428,13 @@
       <c r="E143" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F143" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G143" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H143" s="4" t="n">
+      <c r="F143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I143" s="6" t="n">
@@ -8463,13 +8463,13 @@
       <c r="E144" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F144" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G144" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H144" s="4" t="n">
+      <c r="F144" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G144" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I144" s="6" t="n">
@@ -8498,13 +8498,13 @@
       <c r="E145" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F145" s="4" t="n">
+      <c r="F145" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="G145" s="4" t="n">
+      <c r="G145" s="5" t="n">
         <v>0.0556</v>
       </c>
-      <c r="H145" s="4" t="n">
+      <c r="H145" s="5" t="n">
         <v>0.6</v>
       </c>
       <c r="I145" s="6" t="n">
@@ -8535,13 +8535,13 @@
       <c r="E146" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F146" s="4" t="n">
+      <c r="F146" s="5" t="n">
         <v>0.3333</v>
       </c>
-      <c r="G146" s="4" t="n">
+      <c r="G146" s="5" t="n">
         <v>0.0833</v>
       </c>
-      <c r="H146" s="4" t="n">
+      <c r="H146" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I146" s="6" t="n">
@@ -8636,13 +8636,13 @@
       <c r="E150" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F150" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G150" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H150" s="4" t="n">
+      <c r="F150" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I150" s="6" t="n">
@@ -8671,13 +8671,13 @@
       <c r="E151" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F151" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G151" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H151" s="4" t="n">
+      <c r="F151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I151" s="6" t="n">
@@ -8706,13 +8706,13 @@
       <c r="E152" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F152" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G152" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H152" s="4" t="n">
+      <c r="F152" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I152" s="6" t="n">
@@ -8741,13 +8741,13 @@
       <c r="E153" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F153" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G153" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H153" s="4" t="n">
+      <c r="F153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I153" s="6" t="n">
@@ -8776,13 +8776,13 @@
       <c r="E154" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F154" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G154" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H154" s="4" t="n">
+      <c r="F154" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I154" s="6" t="n">
@@ -8811,13 +8811,13 @@
       <c r="E155" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F155" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G155" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H155" s="4" t="n">
+      <c r="F155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I155" s="6" t="n">
@@ -8846,13 +8846,13 @@
       <c r="E156" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F156" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G156" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H156" s="4" t="n">
+      <c r="F156" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I156" s="6" t="n">
@@ -8881,13 +8881,13 @@
       <c r="E157" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F157" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G157" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H157" s="4" t="n">
+      <c r="F157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I157" s="6" t="n">
@@ -8916,13 +8916,13 @@
       <c r="E158" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F158" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G158" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H158" s="4" t="n">
+      <c r="F158" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I158" s="6" t="n">
@@ -8953,13 +8953,13 @@
       <c r="E159" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F159" s="4" t="n">
+      <c r="F159" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="G159" s="4" t="n">
+      <c r="G159" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="H159" s="4" t="n">
+      <c r="H159" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I159" s="6" t="n">
@@ -9054,13 +9054,13 @@
       <c r="E163" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F163" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G163" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H163" s="4" t="n">
+      <c r="F163" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G163" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I163" s="6" t="n">
@@ -9089,13 +9089,13 @@
       <c r="E164" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F164" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G164" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H164" s="4" t="n">
+      <c r="F164" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G164" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I164" s="6" t="n">
@@ -9124,13 +9124,13 @@
       <c r="E165" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F165" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G165" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H165" s="4" t="n">
+      <c r="F165" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I165" s="6" t="n">
@@ -9159,13 +9159,13 @@
       <c r="E166" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F166" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G166" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H166" s="4" t="n">
+      <c r="F166" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G166" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H166" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I166" s="6" t="n">
@@ -9194,13 +9194,13 @@
       <c r="E167" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F167" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G167" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H167" s="4" t="n">
+      <c r="F167" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G167" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I167" s="6" t="n">
@@ -9229,13 +9229,13 @@
       <c r="E168" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F168" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G168" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H168" s="4" t="n">
+      <c r="F168" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G168" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I168" s="6" t="n">
@@ -9264,13 +9264,13 @@
       <c r="E169" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F169" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G169" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H169" s="4" t="n">
+      <c r="F169" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G169" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I169" s="6" t="n">
@@ -9299,13 +9299,13 @@
       <c r="E170" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F170" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G170" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H170" s="4" t="n">
+      <c r="F170" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G170" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I170" s="6" t="n">
@@ -9334,13 +9334,13 @@
       <c r="E171" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F171" s="4" t="n">
+      <c r="F171" s="5" t="n">
         <v>0.25</v>
       </c>
-      <c r="G171" s="4" t="n">
+      <c r="G171" s="5" t="n">
         <v>0.0278</v>
       </c>
-      <c r="H171" s="4" t="n">
+      <c r="H171" s="5" t="n">
         <v>0.2</v>
       </c>
       <c r="I171" s="6" t="n">
@@ -9371,13 +9371,13 @@
       <c r="E172" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F172" s="4" t="n">
+      <c r="F172" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G172" s="4" t="n">
+      <c r="G172" s="5" t="n">
         <v>0.125</v>
       </c>
-      <c r="H172" s="4" t="n">
+      <c r="H172" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I172" s="6" t="n">
@@ -9472,13 +9472,13 @@
       <c r="E176" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F176" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G176" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H176" s="4" t="n">
+      <c r="F176" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I176" s="6" t="n">
@@ -9507,13 +9507,13 @@
       <c r="E177" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F177" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G177" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H177" s="4" t="n">
+      <c r="F177" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G177" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I177" s="6" t="n">
@@ -9542,13 +9542,13 @@
       <c r="E178" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F178" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G178" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H178" s="4" t="n">
+      <c r="F178" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G178" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H178" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I178" s="6" t="n">
@@ -9577,13 +9577,13 @@
       <c r="E179" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F179" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G179" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H179" s="4" t="n">
+      <c r="F179" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G179" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H179" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I179" s="6" t="n">
@@ -9612,13 +9612,13 @@
       <c r="E180" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F180" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G180" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H180" s="4" t="n">
+      <c r="F180" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G180" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H180" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I180" s="6" t="n">
@@ -9647,13 +9647,13 @@
       <c r="E181" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F181" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G181" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H181" s="4" t="n">
+      <c r="F181" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G181" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H181" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I181" s="6" t="n">
@@ -9682,13 +9682,13 @@
       <c r="E182" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F182" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G182" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H182" s="4" t="n">
+      <c r="F182" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G182" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H182" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I182" s="6" t="n">
@@ -9717,13 +9717,13 @@
       <c r="E183" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F183" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G183" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H183" s="4" t="n">
+      <c r="F183" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G183" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H183" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I183" s="6" t="n">
@@ -9752,13 +9752,13 @@
       <c r="E184" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F184" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G184" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H184" s="4" t="n">
+      <c r="F184" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G184" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H184" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I184" s="6" t="n">
@@ -9789,13 +9789,13 @@
       <c r="E185" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F185" s="4" t="n">
+      <c r="F185" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="G185" s="4" t="n">
+      <c r="G185" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="H185" s="4" t="n">
+      <c r="H185" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I185" s="6" t="n">

</xml_diff>